<commit_message>
Standings: Dave's new workbook links, Sunday AM Ladies, page watcher, DUPR paused
Dave linked new copies of every standings workbook on merrickinapickle.com
(all but Tuesday Pickle Club), so the 6 AM run had been re-reading the old
files since Oct 7. New share ids in sources.mjs; season ids unchanged.
New league sun-ladies (Player-Rankings-c5tt1flK9ajdUjbxtNYy).

Kenny Jee is listed twice in the new Newbridge workbook; Jay confirmed one
person -> sameNameOnePerson. Games 27030 -> 27040: Elle Mac is now on the
Carpenters roster, so 10 held Oct 8 games resolve (Jay approved). None lost.

vps/standings-page.mjs (+test): the daily run reads the Stats & Standings
page and emails when a standings link there is not in sources.mjs. Reports
only; switching stays Jay's call.

vps/dupr-paused: DUPR now locks other players' ratings in the club list;
the daily reading is skipped while this file exists.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importer/live/standings/Player-Rankings-HnAtFNN1bzW2DuOVGi3K.xlsx
+++ b/importer/live/standings/Player-Rankings-HnAtFNN1bzW2DuOVGi3K.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/E914DC20F5C50B12/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{75271A69-8890-4699-A159-E4A6AD3F0C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{618426AC-D233-4601-9FC5-EAA5BC0F96D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8B7C30F7-3EEA-473A-91FF-B5D63174A421}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F00FA0E0-35F8-4997-80F6-A0D8020722AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Player-Rankings-HnAtFNN1bzW2DuO" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="79">
   <si>
     <t>Rank</t>
   </si>
@@ -49,58 +49,67 @@
     <t>Merrick in a pickle</t>
   </si>
   <si>
+    <t>Josh Judge</t>
+  </si>
+  <si>
+    <t>Angel V</t>
+  </si>
+  <si>
     <t>Michael Spezio</t>
   </si>
   <si>
-    <t>Josh Judge</t>
+    <t>Rex Bunt</t>
   </si>
   <si>
     <t>Noah Hackmack</t>
   </si>
   <si>
-    <t>Angel V</t>
+    <t>Vincent Cusumano</t>
+  </si>
+  <si>
+    <t>Adam Kalyvas</t>
   </si>
   <si>
     <t>Jeff Fein</t>
   </si>
   <si>
+    <t>Mike Breitinger</t>
+  </si>
+  <si>
+    <t>Jeff Hersh</t>
+  </si>
+  <si>
+    <t>Pickle United</t>
+  </si>
+  <si>
+    <t>Jason Vargas</t>
+  </si>
+  <si>
+    <t>John McCormack</t>
+  </si>
+  <si>
+    <t>Adam Stork</t>
+  </si>
+  <si>
     <t>Peter Prochilo</t>
   </si>
   <si>
     <t>BOX PICKLEBALL</t>
   </si>
   <si>
-    <t>Rex Bunt</t>
-  </si>
-  <si>
-    <t>John McCormack</t>
-  </si>
-  <si>
-    <t>Adam Kalyvas</t>
-  </si>
-  <si>
-    <t>Vincent Cusumano</t>
-  </si>
-  <si>
-    <t>Mike Breitinger</t>
-  </si>
-  <si>
-    <t>Adam Stork</t>
-  </si>
-  <si>
-    <t>Jason Vargas</t>
-  </si>
-  <si>
-    <t>Jeff Hersh</t>
-  </si>
-  <si>
-    <t>Pickle United</t>
+    <t>Chris Paolina</t>
   </si>
   <si>
     <t>Stephen Rizzi</t>
   </si>
   <si>
-    <t>Chris Paolina</t>
+    <t>Lauren Glodny</t>
+  </si>
+  <si>
+    <t>Gregg Dickens</t>
+  </si>
+  <si>
+    <t>Nicole Beiner</t>
   </si>
   <si>
     <t>Mark Lazo</t>
@@ -109,10 +118,25 @@
     <t>PxP PC</t>
   </si>
   <si>
-    <t>Lauren Glodny</t>
-  </si>
-  <si>
-    <t>Nicole Beiner</t>
+    <t>Robert Mentz</t>
+  </si>
+  <si>
+    <t>Matthew Lupardo</t>
+  </si>
+  <si>
+    <t>LI-Kick</t>
+  </si>
+  <si>
+    <t>Bethuel Bayawa</t>
+  </si>
+  <si>
+    <t>Glenn Saenz</t>
+  </si>
+  <si>
+    <t>Mikel Strauch</t>
+  </si>
+  <si>
+    <t>Christie Simmons</t>
   </si>
   <si>
     <t>Eran Dekel</t>
@@ -124,28 +148,34 @@
     <t>Gary Kotlyar</t>
   </si>
   <si>
-    <t>Robert Mentz</t>
-  </si>
-  <si>
-    <t>Christie Simmons</t>
+    <t>Adrian Murillo</t>
+  </si>
+  <si>
+    <t>Edward Wahl</t>
+  </si>
+  <si>
+    <t>Kenny Jee</t>
   </si>
   <si>
     <t>Richard Vaselli</t>
   </si>
   <si>
+    <t>Sal Farruggia</t>
+  </si>
+  <si>
+    <t>Paul Ilan</t>
+  </si>
+  <si>
+    <t>Olivia O’Keefe</t>
+  </si>
+  <si>
     <t>Luis Lozano</t>
   </si>
   <si>
-    <t>Olivia O’Keefe</t>
-  </si>
-  <si>
-    <t>Matthew Lupardo</t>
-  </si>
-  <si>
-    <t>LI-Kick</t>
-  </si>
-  <si>
-    <t>Adrian Murillo</t>
+    <t>Rong Tian Yu</t>
+  </si>
+  <si>
+    <t>Jason Pomerantz</t>
   </si>
   <si>
     <t>Kevin Monahan</t>
@@ -154,24 +184,33 @@
     <t>Bill Lynch</t>
   </si>
   <si>
+    <t>Brendan Stephenson</t>
+  </si>
+  <si>
     <t>Daniel Calhoun</t>
   </si>
   <si>
-    <t>Kenny Jee</t>
-  </si>
-  <si>
-    <t>Bethuel Bayawa</t>
+    <t>Erik Deangelis</t>
+  </si>
+  <si>
+    <t>Charles Maione</t>
+  </si>
+  <si>
+    <t>David Huber</t>
   </si>
   <si>
     <t>Alexia Yaziciyan</t>
   </si>
   <si>
-    <t>Charles Maione</t>
-  </si>
-  <si>
     <t>Tom McDonough</t>
   </si>
   <si>
+    <t>Jaime Frand</t>
+  </si>
+  <si>
+    <t>Lori McBride</t>
+  </si>
+  <si>
     <t>Michael Scancarello</t>
   </si>
   <si>
@@ -209,6 +248,15 @@
   </si>
   <si>
     <t>Gold</t>
+  </si>
+  <si>
+    <t>NBI WEDNESDAY NIGHT</t>
+  </si>
+  <si>
+    <t>WEEK 8</t>
+  </si>
+  <si>
+    <t>MERRICK IN A PICKLE</t>
   </si>
 </sst>
 </file>
@@ -218,7 +266,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -354,14 +402,19 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Kristen ITC"/>
-      <family val="4"/>
+      <name val="Georgia Pro Cond Black"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Kermit Extrabold"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -549,13 +602,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF7474"/>
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -736,7 +801,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -751,25 +816,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="18" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="33" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -781,14 +831,39 @@
     <xf numFmtId="10" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="19" fillId="36" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="37" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="18" fillId="37" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1165,355 +1240,323 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65FE1473-45D1-48C7-9DD8-48A014187C19}">
-  <dimension ref="A1:R41"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A317B30-3C65-4F10-B586-709463314FD3}">
+  <dimension ref="A1:R56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="18.140625" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" customWidth="1"/>
-    <col min="13" max="13" width="10.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="15" max="15" width="9.140625" style="14"/>
     <col min="17" max="17" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="8" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:18" s="16" customFormat="1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="17"/>
+      <c r="B1" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="O1" s="18"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="17"/>
+    </row>
+    <row r="2" spans="1:18" s="15" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
+      <c r="B2" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E2" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F2" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="K1" s="6" t="s">
+      <c r="G2" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="H2" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="I2" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="J2" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="K2" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="N1" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q1" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="R1" s="6" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="9">
-        <v>104</v>
-      </c>
-      <c r="E2" s="9">
-        <v>35</v>
-      </c>
-      <c r="F2" s="1">
-        <v>20</v>
-      </c>
-      <c r="G2" s="9">
-        <v>55</v>
-      </c>
-      <c r="H2" s="9">
-        <v>591</v>
-      </c>
-      <c r="I2" s="1">
-        <v>525</v>
-      </c>
-      <c r="J2" s="9">
-        <v>66</v>
-      </c>
-      <c r="K2" s="15">
-        <v>0.63600000000000001</v>
-      </c>
-      <c r="L2" s="9">
-        <v>5</v>
-      </c>
-      <c r="M2" s="9">
-        <v>3</v>
-      </c>
-      <c r="N2" s="1">
-        <v>1</v>
-      </c>
-      <c r="O2" s="16">
-        <f>D2/L2</f>
-        <v>20.8</v>
-      </c>
-      <c r="P2" s="9">
-        <v>5</v>
-      </c>
-      <c r="Q2" s="13">
-        <f>P2/L2</f>
-        <v>1</v>
-      </c>
-      <c r="R2" s="9">
-        <v>2</v>
+      <c r="L2" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="M2" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="N2" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="O2" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="P2" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q2" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="R2" s="20" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>9</v>
+        <v>1</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="14">
-        <v>89</v>
-      </c>
-      <c r="E3" s="17">
-        <v>30</v>
+      <c r="D3" s="6">
+        <v>167</v>
+      </c>
+      <c r="E3" s="6">
+        <v>54</v>
       </c>
       <c r="F3" s="1">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G3" s="9">
-        <v>55</v>
-      </c>
-      <c r="H3" s="14">
-        <v>539</v>
+        <v>87</v>
+      </c>
+      <c r="H3" s="6">
+        <v>934</v>
       </c>
       <c r="I3" s="1">
-        <v>541</v>
-      </c>
-      <c r="J3" s="1">
-        <v>-2</v>
+        <v>828</v>
+      </c>
+      <c r="J3" s="6">
+        <v>106</v>
       </c>
       <c r="K3" s="2">
-        <v>0.54500000000000004</v>
-      </c>
-      <c r="L3" s="9">
+        <v>0.621</v>
+      </c>
+      <c r="L3" s="6">
+        <v>8</v>
+      </c>
+      <c r="M3" s="6">
         <v>5</v>
       </c>
-      <c r="M3" s="17">
-        <v>2</v>
-      </c>
       <c r="N3" s="1">
-        <v>2</v>
-      </c>
-      <c r="O3" s="11">
-        <f t="shared" ref="O3:O41" si="0">D3/L3</f>
-        <v>17.8</v>
-      </c>
-      <c r="P3" s="9">
-        <v>5</v>
-      </c>
-      <c r="Q3" s="13">
-        <f t="shared" ref="Q3:Q41" si="1">P3/L3</f>
-        <v>1</v>
-      </c>
-      <c r="R3" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="O3" s="13">
+        <f>D3/L3</f>
+        <v>20.875</v>
+      </c>
+      <c r="P3" s="6">
+        <v>8</v>
+      </c>
+      <c r="Q3" s="8">
+        <f>P3/L3</f>
+        <v>1</v>
+      </c>
+      <c r="R3" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="9">
+        <v>150</v>
+      </c>
+      <c r="E4" s="9">
+        <v>50</v>
+      </c>
+      <c r="F4" s="1">
+        <v>26</v>
+      </c>
+      <c r="G4" s="1">
+        <v>76</v>
+      </c>
+      <c r="H4" s="1">
+        <v>794</v>
+      </c>
+      <c r="I4" s="1">
+        <v>728</v>
+      </c>
+      <c r="J4" s="1">
+        <v>66</v>
+      </c>
+      <c r="K4" s="10">
+        <v>0.65800000000000003</v>
+      </c>
+      <c r="L4" s="1">
+        <v>7</v>
+      </c>
+      <c r="M4" s="6">
+        <v>5</v>
+      </c>
+      <c r="N4" s="1">
+        <v>1</v>
+      </c>
+      <c r="O4" s="13">
+        <f t="shared" ref="O4:O56" si="0">D4/L4</f>
+        <v>21.428571428571427</v>
+      </c>
+      <c r="P4" s="1">
+        <v>7</v>
+      </c>
+      <c r="Q4" s="8">
+        <f t="shared" ref="Q4:Q34" si="1">P4/L4</f>
+        <v>1</v>
+      </c>
+      <c r="R4" s="6">
         <v>3</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="17">
-        <v>87</v>
-      </c>
-      <c r="E4" s="17">
-        <v>30</v>
-      </c>
-      <c r="F4" s="1">
-        <v>14</v>
-      </c>
-      <c r="G4" s="1">
-        <v>44</v>
-      </c>
-      <c r="H4" s="1">
-        <v>464</v>
-      </c>
-      <c r="I4" s="1">
-        <v>426</v>
-      </c>
-      <c r="J4" s="1">
-        <v>38</v>
-      </c>
-      <c r="K4" s="10">
-        <v>0.68200000000000005</v>
-      </c>
-      <c r="L4" s="1">
-        <v>4</v>
-      </c>
-      <c r="M4" s="9">
-        <v>3</v>
-      </c>
-      <c r="N4" s="1">
-        <v>1</v>
-      </c>
-      <c r="O4" s="12">
-        <f t="shared" si="0"/>
-        <v>21.75</v>
-      </c>
-      <c r="P4" s="17">
-        <v>4</v>
-      </c>
-      <c r="Q4" s="13">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="R4" s="9">
-        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="11">
+        <v>140</v>
+      </c>
+      <c r="E5" s="11">
+        <v>49</v>
+      </c>
+      <c r="F5" s="1">
+        <v>28</v>
+      </c>
+      <c r="G5" s="1">
+        <v>77</v>
+      </c>
+      <c r="H5" s="1">
+        <v>828</v>
+      </c>
+      <c r="I5" s="1">
+        <v>758</v>
+      </c>
+      <c r="J5" s="11">
+        <v>70</v>
+      </c>
+      <c r="K5" s="12">
+        <v>0.63600000000000001</v>
+      </c>
+      <c r="L5" s="1">
+        <v>7</v>
+      </c>
+      <c r="M5" s="11">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="1">
-        <v>78</v>
-      </c>
-      <c r="E5" s="1">
-        <v>28</v>
-      </c>
-      <c r="F5" s="1">
-        <v>16</v>
-      </c>
-      <c r="G5" s="1">
-        <v>44</v>
-      </c>
-      <c r="H5" s="1">
-        <v>457</v>
-      </c>
-      <c r="I5" s="1">
-        <v>395</v>
-      </c>
-      <c r="J5" s="14">
-        <v>62</v>
-      </c>
-      <c r="K5" s="15">
-        <v>0.63600000000000001</v>
-      </c>
-      <c r="L5" s="1">
-        <v>4</v>
-      </c>
-      <c r="M5" s="1">
-        <v>1</v>
-      </c>
       <c r="N5" s="1">
         <v>1</v>
       </c>
-      <c r="O5" s="18">
-        <f t="shared" si="0"/>
-        <v>19.5</v>
-      </c>
-      <c r="P5" s="17">
-        <v>4</v>
-      </c>
-      <c r="Q5" s="13">
+      <c r="O5" s="13">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="P5" s="1">
+        <v>7</v>
+      </c>
+      <c r="Q5" s="8">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="R5" s="17">
-        <v>1</v>
+      <c r="R5" s="11">
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="1">
+        <v>123</v>
+      </c>
+      <c r="E6" s="1">
+        <v>41</v>
+      </c>
+      <c r="F6" s="1">
+        <v>35</v>
+      </c>
+      <c r="G6" s="1">
         <v>76</v>
       </c>
-      <c r="E6" s="1">
-        <v>28</v>
-      </c>
-      <c r="F6" s="1">
-        <v>16</v>
-      </c>
-      <c r="G6" s="1">
-        <v>44</v>
-      </c>
       <c r="H6" s="1">
-        <v>472</v>
+        <v>742</v>
       </c>
       <c r="I6" s="1">
-        <v>428</v>
-      </c>
-      <c r="J6" s="17">
-        <v>44</v>
-      </c>
-      <c r="K6" s="15">
-        <v>0.63600000000000001</v>
+        <v>756</v>
+      </c>
+      <c r="J6" s="1">
+        <v>-14</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0.53900000000000003</v>
       </c>
       <c r="L6" s="1">
-        <v>4</v>
-      </c>
-      <c r="M6" s="17">
+        <v>7</v>
+      </c>
+      <c r="M6" s="1">
         <v>2</v>
       </c>
       <c r="N6" s="1">
         <v>2</v>
       </c>
-      <c r="O6" s="11">
-        <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-      <c r="P6" s="17">
-        <v>4</v>
-      </c>
-      <c r="Q6" s="13">
+      <c r="O6" s="13">
+        <f t="shared" si="0"/>
+        <v>17.571428571428573</v>
+      </c>
+      <c r="P6" s="1">
+        <v>7</v>
+      </c>
+      <c r="Q6" s="8">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -1524,332 +1567,334 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="1">
-        <v>76</v>
+        <v>122</v>
       </c>
       <c r="E7" s="1">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="F7" s="1">
-        <v>28</v>
-      </c>
-      <c r="G7" s="9">
-        <v>55</v>
-      </c>
-      <c r="H7" s="1">
-        <v>540</v>
+        <v>40</v>
+      </c>
+      <c r="G7" s="1">
+        <v>85</v>
+      </c>
+      <c r="H7" s="11">
+        <v>854</v>
       </c>
       <c r="I7" s="1">
-        <v>532</v>
+        <v>832</v>
       </c>
       <c r="J7" s="1">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="K7" s="2">
-        <v>0.49099999999999999</v>
-      </c>
-      <c r="L7" s="9">
-        <v>5</v>
+        <v>0.52900000000000003</v>
+      </c>
+      <c r="L7" s="6">
+        <v>8</v>
       </c>
       <c r="M7" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N7" s="1">
-        <v>3</v>
-      </c>
-      <c r="O7" s="11">
-        <f t="shared" si="0"/>
-        <v>15.2</v>
-      </c>
-      <c r="P7" s="17">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="O7" s="13">
+        <f t="shared" si="0"/>
+        <v>15.25</v>
+      </c>
+      <c r="P7" s="1">
+        <v>6</v>
       </c>
       <c r="Q7" s="4">
         <f t="shared" si="1"/>
-        <v>0.8</v>
-      </c>
-      <c r="R7" s="1"/>
+        <v>0.75</v>
+      </c>
+      <c r="R7" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D8" s="1">
-        <v>74</v>
+        <v>120</v>
       </c>
       <c r="E8" s="1">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="F8" s="1">
-        <v>31</v>
-      </c>
-      <c r="G8" s="9">
-        <v>55</v>
+        <v>22</v>
+      </c>
+      <c r="G8" s="1">
+        <v>66</v>
       </c>
       <c r="H8" s="1">
-        <v>531</v>
+        <v>681</v>
       </c>
       <c r="I8" s="1">
-        <v>547</v>
-      </c>
-      <c r="J8" s="1">
-        <v>-16</v>
-      </c>
-      <c r="K8" s="2">
-        <v>0.436</v>
-      </c>
-      <c r="L8" s="9">
-        <v>5</v>
+        <v>578</v>
+      </c>
+      <c r="J8" s="9">
+        <v>103</v>
+      </c>
+      <c r="K8" s="7">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="L8" s="1">
+        <v>6</v>
       </c>
       <c r="M8" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N8" s="1">
-        <v>4</v>
-      </c>
-      <c r="O8" s="11">
-        <f t="shared" si="0"/>
-        <v>14.8</v>
-      </c>
-      <c r="P8" s="17">
-        <v>4</v>
-      </c>
-      <c r="Q8" s="4">
+        <v>1</v>
+      </c>
+      <c r="O8" s="13">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="P8" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q8" s="8">
         <f t="shared" si="1"/>
-        <v>0.8</v>
-      </c>
-      <c r="R8" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="R8" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="1">
-        <v>74</v>
-      </c>
-      <c r="E9" s="14">
-        <v>31</v>
+        <v>115</v>
+      </c>
+      <c r="E9" s="1">
+        <v>38</v>
       </c>
       <c r="F9" s="1">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="G9" s="1">
-        <v>53</v>
-      </c>
-      <c r="H9" s="14">
-        <v>539</v>
+        <v>76</v>
+      </c>
+      <c r="H9" s="1">
+        <v>762</v>
       </c>
       <c r="I9" s="1">
-        <v>499</v>
+        <v>772</v>
       </c>
       <c r="J9" s="1">
-        <v>40</v>
-      </c>
-      <c r="K9" s="2">
-        <v>0.58499999999999996</v>
-      </c>
-      <c r="L9" s="9">
-        <v>5</v>
-      </c>
-      <c r="M9" s="17">
-        <v>2</v>
+        <v>-10</v>
+      </c>
+      <c r="K9" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="L9" s="1">
+        <v>7</v>
+      </c>
+      <c r="M9" s="1">
+        <v>0</v>
       </c>
       <c r="N9" s="1">
-        <v>1</v>
-      </c>
-      <c r="O9" s="11">
-        <f t="shared" si="0"/>
-        <v>14.8</v>
+        <v>4</v>
+      </c>
+      <c r="O9" s="13">
+        <f t="shared" si="0"/>
+        <v>16.428571428571427</v>
       </c>
       <c r="P9" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q9" s="4">
         <f t="shared" si="1"/>
-        <v>0.6</v>
-      </c>
-      <c r="R9" s="17">
-        <v>1</v>
-      </c>
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="R9" s="1"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="1">
-        <v>72</v>
+        <v>109</v>
       </c>
       <c r="E10" s="1">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="F10" s="1">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="G10" s="9">
-        <v>55</v>
-      </c>
-      <c r="H10" s="1">
-        <v>536</v>
+        <v>87</v>
+      </c>
+      <c r="H10" s="9">
+        <v>866</v>
       </c>
       <c r="I10" s="1">
-        <v>533</v>
+        <v>842</v>
       </c>
       <c r="J10" s="1">
+        <v>24</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0.52900000000000003</v>
+      </c>
+      <c r="L10" s="6">
+        <v>8</v>
+      </c>
+      <c r="M10" s="1">
         <v>3</v>
       </c>
-      <c r="K10" s="2">
-        <v>0.49099999999999999</v>
-      </c>
-      <c r="L10" s="9">
-        <v>5</v>
-      </c>
-      <c r="M10" s="17">
+      <c r="N10" s="1">
         <v>2</v>
       </c>
-      <c r="N10" s="1">
-        <v>3</v>
-      </c>
-      <c r="O10" s="11">
-        <f t="shared" si="0"/>
-        <v>14.4</v>
+      <c r="O10" s="13">
+        <f t="shared" si="0"/>
+        <v>13.625</v>
       </c>
       <c r="P10" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="4">
         <f t="shared" si="1"/>
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="R10" s="1"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="1">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="E11" s="1">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="F11" s="1">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="G11" s="1">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="H11" s="1">
-        <v>532</v>
+        <v>743</v>
       </c>
       <c r="I11" s="1">
-        <v>514</v>
+        <v>772</v>
       </c>
       <c r="J11" s="1">
-        <v>18</v>
+        <v>-29</v>
       </c>
       <c r="K11" s="2">
-        <v>0.51900000000000002</v>
-      </c>
-      <c r="L11" s="9">
-        <v>5</v>
-      </c>
-      <c r="M11" s="17">
-        <v>2</v>
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="L11" s="1">
+        <v>7</v>
+      </c>
+      <c r="M11" s="1">
+        <v>1</v>
       </c>
       <c r="N11" s="1">
-        <v>2</v>
-      </c>
-      <c r="O11" s="11">
-        <f t="shared" si="0"/>
-        <v>14.2</v>
+        <v>3</v>
+      </c>
+      <c r="O11" s="13">
+        <f t="shared" si="0"/>
+        <v>15.285714285714286</v>
       </c>
       <c r="P11" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q11" s="4">
         <f t="shared" si="1"/>
-        <v>0.6</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="R11" s="1"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="1">
-        <v>70</v>
+        <v>102</v>
       </c>
       <c r="E12" s="1">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="F12" s="1">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="G12" s="1">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="H12" s="1">
-        <v>456</v>
+        <v>682</v>
       </c>
       <c r="I12" s="1">
-        <v>445</v>
+        <v>669</v>
       </c>
       <c r="J12" s="1">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K12" s="2">
-        <v>0.54500000000000004</v>
+        <v>0.51500000000000001</v>
       </c>
       <c r="L12" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M12" s="1">
         <v>0</v>
       </c>
       <c r="N12" s="1">
-        <v>4</v>
-      </c>
-      <c r="O12" s="11">
-        <f t="shared" si="0"/>
-        <v>17.5</v>
-      </c>
-      <c r="P12" s="17">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="O12" s="13">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="P12" s="1">
+        <v>6</v>
       </c>
       <c r="Q12" s="4">
         <f t="shared" si="1"/>
@@ -1859,317 +1904,324 @@
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D13" s="1">
-        <v>69</v>
+        <v>101</v>
       </c>
       <c r="E13" s="1">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="F13" s="1">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G13" s="1">
-        <v>44</v>
+        <v>76</v>
       </c>
       <c r="H13" s="1">
-        <v>478</v>
+        <v>778</v>
       </c>
       <c r="I13" s="1">
-        <v>458</v>
+        <v>739</v>
       </c>
       <c r="J13" s="1">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="K13" s="2">
-        <v>0.56799999999999995</v>
+        <v>0.57899999999999996</v>
       </c>
       <c r="L13" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M13" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N13" s="1">
-        <v>5</v>
-      </c>
-      <c r="O13" s="11">
-        <f t="shared" si="0"/>
-        <v>17.25</v>
-      </c>
-      <c r="P13" s="17">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="O13" s="13">
+        <f t="shared" si="0"/>
+        <v>14.428571428571429</v>
+      </c>
+      <c r="P13" s="1">
+        <v>6</v>
       </c>
       <c r="Q13" s="4">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="R13" s="1"/>
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="R13" s="1">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="1">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="E14" s="1">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="F14" s="1">
-        <v>28</v>
-      </c>
-      <c r="G14" s="1">
-        <v>54</v>
+        <v>49</v>
+      </c>
+      <c r="G14" s="6">
+        <v>88</v>
       </c>
       <c r="H14" s="1">
-        <v>513</v>
+        <v>844</v>
       </c>
       <c r="I14" s="1">
-        <v>532</v>
+        <v>886</v>
       </c>
       <c r="J14" s="1">
-        <v>-19</v>
+        <v>-42</v>
       </c>
       <c r="K14" s="2">
-        <v>0.48099999999999998</v>
-      </c>
-      <c r="L14" s="9">
-        <v>5</v>
+        <v>0.443</v>
+      </c>
+      <c r="L14" s="6">
+        <v>8</v>
       </c>
       <c r="M14" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N14" s="1">
+        <v>1</v>
+      </c>
+      <c r="O14" s="13">
+        <f t="shared" si="0"/>
+        <v>12.5</v>
+      </c>
+      <c r="P14" s="1">
         <v>4</v>
-      </c>
-      <c r="O14" s="11">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="P14" s="1">
-        <v>3</v>
       </c>
       <c r="Q14" s="4">
         <f t="shared" si="1"/>
-        <v>0.6</v>
-      </c>
-      <c r="R14" s="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="R14" s="1">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="1">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="E15" s="1">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F15" s="1">
-        <v>31</v>
-      </c>
-      <c r="G15" s="9">
-        <v>55</v>
+        <v>36</v>
+      </c>
+      <c r="G15" s="1">
+        <v>66</v>
       </c>
       <c r="H15" s="1">
-        <v>520</v>
+        <v>638</v>
       </c>
       <c r="I15" s="1">
-        <v>545</v>
+        <v>645</v>
       </c>
       <c r="J15" s="1">
-        <v>-25</v>
+        <v>-7</v>
       </c>
       <c r="K15" s="2">
-        <v>0.436</v>
-      </c>
-      <c r="L15" s="9">
-        <v>5</v>
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="L15" s="1">
+        <v>6</v>
       </c>
       <c r="M15" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N15" s="1">
-        <v>1</v>
-      </c>
-      <c r="O15" s="11">
-        <f t="shared" si="0"/>
-        <v>12.8</v>
+        <v>3</v>
+      </c>
+      <c r="O15" s="13">
+        <f t="shared" si="0"/>
+        <v>14.5</v>
       </c>
       <c r="P15" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q15" s="4">
         <f t="shared" si="1"/>
-        <v>0.6</v>
-      </c>
-      <c r="R15" s="1">
-        <v>0.5</v>
-      </c>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="R15" s="1"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="D16" s="1">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="E16" s="1">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F16" s="1">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="G16" s="1">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="H16" s="1">
-        <v>438</v>
+        <v>614</v>
       </c>
       <c r="I16" s="1">
-        <v>422</v>
+        <v>650</v>
       </c>
       <c r="J16" s="1">
-        <v>16</v>
+        <v>-36</v>
       </c>
       <c r="K16" s="2">
-        <v>0.53500000000000003</v>
+        <v>0.44600000000000001</v>
       </c>
       <c r="L16" s="1">
+        <v>6</v>
+      </c>
+      <c r="M16" s="1">
+        <v>0</v>
+      </c>
+      <c r="N16" s="1">
         <v>4</v>
       </c>
-      <c r="M16" s="1">
-        <v>2</v>
-      </c>
-      <c r="N16" s="1">
-        <v>2</v>
-      </c>
-      <c r="O16" s="11">
-        <f t="shared" si="0"/>
-        <v>12.75</v>
-      </c>
-      <c r="P16" s="1"/>
-      <c r="Q16" s="4"/>
+      <c r="O16" s="13">
+        <f t="shared" si="0"/>
+        <v>13.166666666666666</v>
+      </c>
+      <c r="P16" s="1">
+        <v>4</v>
+      </c>
+      <c r="Q16" s="4">
+        <f t="shared" si="1"/>
+        <v>0.66666666666666663</v>
+      </c>
       <c r="R16" s="1"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="D17" s="1">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="E17" s="1">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F17" s="1">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G17" s="1">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H17" s="1">
-        <v>438</v>
+        <v>531</v>
       </c>
       <c r="I17" s="1">
-        <v>448</v>
+        <v>547</v>
       </c>
       <c r="J17" s="1">
-        <v>-10</v>
+        <v>-16</v>
       </c>
       <c r="K17" s="2">
-        <v>0.432</v>
+        <v>0.436</v>
       </c>
       <c r="L17" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M17" s="1">
         <v>0</v>
       </c>
       <c r="N17" s="1">
-        <v>7</v>
-      </c>
-      <c r="O17" s="11">
-        <f t="shared" si="0"/>
-        <v>12</v>
+        <v>4</v>
+      </c>
+      <c r="O17" s="13">
+        <f t="shared" si="0"/>
+        <v>14.8</v>
       </c>
       <c r="P17" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q17" s="4">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="R17" s="1"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="1">
+        <v>71</v>
+      </c>
+      <c r="E18" s="1">
         <v>26</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="1">
-        <v>46</v>
-      </c>
-      <c r="E18" s="1">
-        <v>19</v>
-      </c>
       <c r="F18" s="1">
-        <v>35</v>
-      </c>
-      <c r="G18" s="1">
-        <v>54</v>
+        <v>61</v>
+      </c>
+      <c r="G18" s="9">
+        <v>87</v>
       </c>
       <c r="H18" s="1">
-        <v>469</v>
+        <v>751</v>
       </c>
       <c r="I18" s="1">
-        <v>568</v>
+        <v>922</v>
       </c>
       <c r="J18" s="1">
-        <v>-99</v>
+        <v>-171</v>
       </c>
       <c r="K18" s="2">
-        <v>0.35199999999999998</v>
-      </c>
-      <c r="L18" s="9">
-        <v>5</v>
+        <v>0.29899999999999999</v>
+      </c>
+      <c r="L18" s="6">
+        <v>8</v>
       </c>
       <c r="M18" s="1">
         <v>0</v>
@@ -2177,106 +2229,111 @@
       <c r="N18" s="1">
         <v>6</v>
       </c>
-      <c r="O18" s="11">
-        <f t="shared" si="0"/>
-        <v>9.1999999999999993</v>
+      <c r="O18" s="13">
+        <f t="shared" si="0"/>
+        <v>8.875</v>
       </c>
       <c r="P18" s="1">
         <v>1</v>
       </c>
       <c r="Q18" s="4">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>0.125</v>
       </c>
       <c r="R18" s="1"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D19" s="1">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="E19" s="1">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F19" s="1">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="G19" s="1">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="H19" s="1">
-        <v>359</v>
+        <v>655</v>
       </c>
       <c r="I19" s="1">
-        <v>315</v>
+        <v>639</v>
       </c>
       <c r="J19" s="1">
-        <v>44</v>
-      </c>
-      <c r="K19" s="2">
-        <v>0.60599999999999998</v>
+        <v>16</v>
+      </c>
+      <c r="K19" s="3">
+        <v>0.47</v>
       </c>
       <c r="L19" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M19" s="1">
+        <v>0</v>
+      </c>
+      <c r="N19" s="1">
+        <v>5</v>
+      </c>
+      <c r="O19" s="13">
+        <f t="shared" si="0"/>
+        <v>11.666666666666666</v>
+      </c>
+      <c r="P19" s="1">
         <v>2</v>
       </c>
-      <c r="N19" s="1">
-        <v>2</v>
-      </c>
-      <c r="O19" s="11">
-        <f t="shared" si="0"/>
-        <v>13.333333333333334</v>
-      </c>
-      <c r="P19" s="1"/>
-      <c r="Q19" s="4"/>
+      <c r="Q19" s="4">
+        <f t="shared" si="1"/>
+        <v>0.33333333333333331</v>
+      </c>
       <c r="R19" s="1"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="1">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="E20" s="1">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F20" s="1">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="G20" s="1">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="H20" s="1">
-        <v>380</v>
+        <v>686</v>
       </c>
       <c r="I20" s="1">
-        <v>452</v>
+        <v>768</v>
       </c>
       <c r="J20" s="1">
-        <v>-72</v>
+        <v>-82</v>
       </c>
       <c r="K20" s="2">
-        <v>0.372</v>
+        <v>0.39500000000000002</v>
       </c>
       <c r="L20" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M20" s="1">
         <v>0</v>
@@ -2284,9 +2341,9 @@
       <c r="N20" s="1">
         <v>5</v>
       </c>
-      <c r="O20" s="11">
-        <f t="shared" si="0"/>
-        <v>9.75</v>
+      <c r="O20" s="13">
+        <f t="shared" si="0"/>
+        <v>9.8571428571428577</v>
       </c>
       <c r="P20" s="1"/>
       <c r="Q20" s="4"/>
@@ -2294,282 +2351,279 @@
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D21" s="1">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="E21" s="1">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F21" s="1">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="G21" s="1">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="H21" s="1">
-        <v>391</v>
+        <v>325</v>
       </c>
       <c r="I21" s="1">
-        <v>447</v>
+        <v>312</v>
       </c>
       <c r="J21" s="1">
-        <v>-56</v>
+        <v>13</v>
       </c>
       <c r="K21" s="2">
-        <v>0.32600000000000001</v>
+        <v>0.53100000000000003</v>
       </c>
       <c r="L21" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M21" s="1">
         <v>0</v>
       </c>
       <c r="N21" s="1">
-        <v>9</v>
-      </c>
-      <c r="O21" s="11">
-        <f t="shared" si="0"/>
-        <v>8.75</v>
-      </c>
-      <c r="P21" s="1">
-        <v>1</v>
-      </c>
-      <c r="Q21" s="4">
-        <f t="shared" si="1"/>
-        <v>0.25</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="O21" s="13">
+        <f t="shared" si="0"/>
+        <v>16.666666666666668</v>
+      </c>
+      <c r="P21" s="1"/>
+      <c r="Q21" s="4"/>
       <c r="R21" s="1"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="1">
+        <v>49</v>
+      </c>
+      <c r="E22" s="1">
+        <v>23</v>
+      </c>
+      <c r="F22" s="1">
         <v>31</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="1">
-        <v>31</v>
-      </c>
-      <c r="E22" s="1">
-        <v>10</v>
-      </c>
-      <c r="F22" s="1">
-        <v>12</v>
-      </c>
       <c r="G22" s="1">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="H22" s="1">
-        <v>200</v>
+        <v>512</v>
       </c>
       <c r="I22" s="1">
-        <v>198</v>
+        <v>536</v>
       </c>
       <c r="J22" s="1">
-        <v>2</v>
+        <v>-24</v>
       </c>
       <c r="K22" s="2">
-        <v>0.45500000000000002</v>
+        <v>0.42599999999999999</v>
       </c>
       <c r="L22" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M22" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" s="1">
-        <v>9</v>
-      </c>
-      <c r="O22" s="11">
-        <f t="shared" si="0"/>
-        <v>15.5</v>
+        <v>1</v>
+      </c>
+      <c r="O22" s="13">
+        <f t="shared" si="0"/>
+        <v>9.8000000000000007</v>
       </c>
       <c r="P22" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q22" s="4">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="R22" s="1"/>
+        <v>0.2</v>
+      </c>
+      <c r="R22" s="1">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="D23" s="1">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="E23" s="1">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F23" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G23" s="1">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="H23" s="1">
-        <v>300</v>
+        <v>459</v>
       </c>
       <c r="I23" s="1">
-        <v>315</v>
+        <v>434</v>
       </c>
       <c r="J23" s="1">
-        <v>-15</v>
+        <v>25</v>
       </c>
       <c r="K23" s="2">
-        <v>0.40600000000000003</v>
+        <v>0.54500000000000004</v>
       </c>
       <c r="L23" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M23" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N23" s="1">
-        <v>5</v>
-      </c>
-      <c r="O23" s="11">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="P23" s="1">
-        <v>1</v>
-      </c>
-      <c r="Q23" s="4">
-        <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O23" s="13">
+        <f t="shared" si="0"/>
+        <v>12.25</v>
+      </c>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="4"/>
       <c r="R23" s="1"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D24" s="1">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="E24" s="1">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F24" s="1">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="G24" s="1">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="H24" s="1">
-        <v>224</v>
+        <v>452</v>
       </c>
       <c r="I24" s="1">
-        <v>233</v>
+        <v>565</v>
       </c>
       <c r="J24" s="1">
-        <v>-9</v>
+        <v>-113</v>
       </c>
       <c r="K24" s="2">
-        <v>0.45500000000000002</v>
+        <v>0.25900000000000001</v>
       </c>
       <c r="L24" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M24" s="1">
         <v>0</v>
       </c>
       <c r="N24" s="1">
-        <v>9</v>
-      </c>
-      <c r="O24" s="11">
-        <f t="shared" si="0"/>
-        <v>14.5</v>
-      </c>
-      <c r="P24" s="1"/>
-      <c r="Q24" s="4"/>
+        <v>7</v>
+      </c>
+      <c r="O24" s="13">
+        <f t="shared" si="0"/>
+        <v>8.4</v>
+      </c>
+      <c r="P24" s="1">
+        <v>1</v>
+      </c>
+      <c r="Q24" s="4">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
       <c r="R24" s="1"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
+        <v>23</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" s="1">
+        <v>41</v>
+      </c>
+      <c r="E25" s="1">
         <v>24</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="1">
-        <v>27</v>
-      </c>
-      <c r="E25" s="1">
-        <v>10</v>
-      </c>
       <c r="F25" s="1">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G25" s="1">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="H25" s="1">
-        <v>263</v>
+        <v>440</v>
       </c>
       <c r="I25" s="1">
-        <v>324</v>
+        <v>464</v>
       </c>
       <c r="J25" s="1">
-        <v>-61</v>
+        <v>-24</v>
       </c>
       <c r="K25" s="2">
-        <v>0.313</v>
+        <v>0.54500000000000004</v>
       </c>
       <c r="L25" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M25" s="1">
+        <v>1</v>
+      </c>
+      <c r="N25" s="1">
+        <v>2</v>
+      </c>
+      <c r="O25" s="13">
+        <f t="shared" si="0"/>
+        <v>10.25</v>
+      </c>
+      <c r="P25" s="1">
         <v>0</v>
-      </c>
-      <c r="N25" s="1">
-        <v>7</v>
-      </c>
-      <c r="O25" s="11">
-        <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="P25" s="1">
-        <v>1</v>
       </c>
       <c r="Q25" s="4">
         <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
+        <v>0</v>
       </c>
       <c r="R25" s="1"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>35</v>
@@ -2578,54 +2632,51 @@
         <v>8</v>
       </c>
       <c r="D26" s="1">
+        <v>37</v>
+      </c>
+      <c r="E26" s="1">
         <v>23</v>
       </c>
-      <c r="E26" s="1">
-        <v>12</v>
-      </c>
       <c r="F26" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G26" s="1">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="H26" s="1">
-        <v>209</v>
+        <v>333</v>
       </c>
       <c r="I26" s="1">
-        <v>198</v>
+        <v>293</v>
       </c>
       <c r="J26" s="1">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="K26" s="2">
-        <v>0.57099999999999995</v>
+        <v>0.69699999999999995</v>
       </c>
       <c r="L26" s="1">
+        <v>3</v>
+      </c>
+      <c r="M26" s="1">
         <v>2</v>
       </c>
-      <c r="M26" s="1">
-        <v>0</v>
-      </c>
       <c r="N26" s="1">
-        <v>4</v>
-      </c>
-      <c r="O26" s="11">
-        <f t="shared" si="0"/>
-        <v>11.5</v>
-      </c>
-      <c r="P26" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R26" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="O26" s="13">
+        <f t="shared" si="0"/>
+        <v>12.333333333333334</v>
+      </c>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="4"/>
+      <c r="R26" s="1">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>36</v>
@@ -2634,41 +2685,41 @@
         <v>8</v>
       </c>
       <c r="D27" s="1">
+        <v>34</v>
+      </c>
+      <c r="E27" s="1">
+        <v>10</v>
+      </c>
+      <c r="F27" s="1">
+        <v>11</v>
+      </c>
+      <c r="G27" s="1">
         <v>21</v>
       </c>
-      <c r="E27" s="1">
-        <v>8</v>
-      </c>
-      <c r="F27" s="1">
-        <v>3</v>
-      </c>
-      <c r="G27" s="1">
-        <v>11</v>
-      </c>
       <c r="H27" s="1">
-        <v>119</v>
+        <v>204</v>
       </c>
       <c r="I27" s="1">
-        <v>92</v>
+        <v>208</v>
       </c>
       <c r="J27" s="1">
-        <v>27</v>
+        <v>-4</v>
       </c>
       <c r="K27" s="2">
-        <v>0.72699999999999998</v>
+        <v>0.47599999999999998</v>
       </c>
       <c r="L27" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M27" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N27" s="1">
-        <v>2</v>
-      </c>
-      <c r="O27" s="11">
-        <f t="shared" si="0"/>
-        <v>21</v>
+        <v>4</v>
+      </c>
+      <c r="O27" s="13">
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
       <c r="P27" s="1"/>
       <c r="Q27" s="4"/>
@@ -2676,7 +2727,7 @@
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>37</v>
@@ -2685,49 +2736,54 @@
         <v>8</v>
       </c>
       <c r="D28" s="1">
+        <v>31</v>
+      </c>
+      <c r="E28" s="1">
         <v>17</v>
       </c>
-      <c r="E28" s="1">
-        <v>6</v>
-      </c>
       <c r="F28" s="1">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="G28" s="1">
+        <v>33</v>
+      </c>
+      <c r="H28" s="1">
+        <v>333</v>
+      </c>
+      <c r="I28" s="1">
+        <v>322</v>
+      </c>
+      <c r="J28" s="1">
         <v>11</v>
       </c>
-      <c r="H28" s="1">
-        <v>110</v>
-      </c>
-      <c r="I28" s="1">
-        <v>82</v>
-      </c>
-      <c r="J28" s="1">
-        <v>28</v>
-      </c>
       <c r="K28" s="2">
-        <v>0.54500000000000004</v>
+        <v>0.51500000000000001</v>
       </c>
       <c r="L28" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M28" s="1">
+        <v>1</v>
+      </c>
+      <c r="N28" s="1">
+        <v>2</v>
+      </c>
+      <c r="O28" s="13">
+        <f t="shared" si="0"/>
+        <v>10.333333333333334</v>
+      </c>
+      <c r="P28" s="1">
         <v>0</v>
       </c>
-      <c r="N28" s="1">
-        <v>6</v>
-      </c>
-      <c r="O28" s="11">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="P28" s="1"/>
-      <c r="Q28" s="4"/>
+      <c r="Q28" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R28" s="1"/>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>38</v>
@@ -2736,64 +2792,69 @@
         <v>8</v>
       </c>
       <c r="D29" s="1">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E29" s="1">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F29" s="1">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G29" s="1">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="H29" s="1">
-        <v>209</v>
+        <v>304</v>
       </c>
       <c r="I29" s="1">
-        <v>232</v>
+        <v>322</v>
       </c>
       <c r="J29" s="1">
-        <v>-23</v>
+        <v>-18</v>
       </c>
       <c r="K29" s="2">
-        <v>0.27300000000000002</v>
+        <v>0.40600000000000003</v>
       </c>
       <c r="L29" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M29" s="1">
         <v>0</v>
       </c>
       <c r="N29" s="1">
-        <v>9</v>
-      </c>
-      <c r="O29" s="11">
-        <f t="shared" si="0"/>
-        <v>8.5</v>
-      </c>
-      <c r="P29" s="1"/>
-      <c r="Q29" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="O29" s="13">
+        <f t="shared" si="0"/>
+        <v>10.333333333333334</v>
+      </c>
+      <c r="P29" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R29" s="1"/>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>39</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="D30" s="1">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="E30" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F30" s="1">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G30" s="1">
         <v>22</v>
@@ -2802,13 +2863,13 @@
         <v>200</v>
       </c>
       <c r="I30" s="1">
-        <v>243</v>
+        <v>198</v>
       </c>
       <c r="J30" s="1">
-        <v>-43</v>
+        <v>2</v>
       </c>
       <c r="K30" s="2">
-        <v>0.36399999999999999</v>
+        <v>0.45500000000000002</v>
       </c>
       <c r="L30" s="1">
         <v>2</v>
@@ -2817,70 +2878,75 @@
         <v>0</v>
       </c>
       <c r="N30" s="1">
-        <v>11</v>
-      </c>
-      <c r="O30" s="11">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="O30" s="13">
+        <f t="shared" si="0"/>
+        <v>15.5</v>
       </c>
       <c r="P30" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="4">
+        <v>2</v>
+      </c>
+      <c r="Q30" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R30" s="1"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
+        <v>29</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" s="1">
         <v>30</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D31" s="1">
-        <v>14</v>
-      </c>
       <c r="E31" s="1">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="F31" s="1">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="G31" s="1">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="H31" s="1">
-        <v>105</v>
+        <v>300</v>
       </c>
       <c r="I31" s="1">
-        <v>127</v>
+        <v>315</v>
       </c>
       <c r="J31" s="1">
-        <v>-22</v>
+        <v>-15</v>
       </c>
       <c r="K31" s="2">
-        <v>0.182</v>
+        <v>0.40600000000000003</v>
       </c>
       <c r="L31" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M31" s="1">
         <v>0</v>
       </c>
       <c r="N31" s="1">
-        <v>12</v>
-      </c>
-      <c r="O31" s="11">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="P31" s="1"/>
-      <c r="Q31" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="O31" s="13">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="P31" s="1">
+        <v>1</v>
+      </c>
+      <c r="Q31" s="4">
+        <f t="shared" si="1"/>
+        <v>0.33333333333333331</v>
+      </c>
       <c r="R31" s="1"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
@@ -2888,98 +2954,96 @@
         <v>30</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D32" s="1">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="E32" s="1">
+        <v>10</v>
+      </c>
+      <c r="F32" s="1">
+        <v>12</v>
+      </c>
+      <c r="G32" s="1">
+        <v>22</v>
+      </c>
+      <c r="H32" s="1">
+        <v>224</v>
+      </c>
+      <c r="I32" s="1">
+        <v>233</v>
+      </c>
+      <c r="J32" s="1">
+        <v>-9</v>
+      </c>
+      <c r="K32" s="2">
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="L32" s="1">
+        <v>2</v>
+      </c>
+      <c r="M32" s="1">
+        <v>0</v>
+      </c>
+      <c r="N32" s="1">
         <v>9</v>
       </c>
-      <c r="F32" s="1">
-        <v>2</v>
-      </c>
-      <c r="G32" s="1">
-        <v>11</v>
-      </c>
-      <c r="H32" s="1">
-        <v>118</v>
-      </c>
-      <c r="I32" s="1">
-        <v>87</v>
-      </c>
-      <c r="J32" s="1">
-        <v>31</v>
-      </c>
-      <c r="K32" s="2">
-        <v>0.81799999999999995</v>
-      </c>
-      <c r="L32" s="1">
-        <v>1</v>
-      </c>
-      <c r="M32" s="1">
-        <v>1</v>
-      </c>
-      <c r="N32" s="1">
-        <v>1</v>
-      </c>
-      <c r="O32" s="11">
-        <f t="shared" si="0"/>
-        <v>14</v>
+      <c r="O32" s="13">
+        <f t="shared" si="0"/>
+        <v>14.5</v>
       </c>
       <c r="P32" s="1"/>
       <c r="Q32" s="4"/>
-      <c r="R32" s="1">
-        <v>0.5</v>
-      </c>
+      <c r="R32" s="1"/>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="D33" s="1">
+        <v>26</v>
+      </c>
+      <c r="E33" s="1">
+        <v>9</v>
+      </c>
+      <c r="F33" s="1">
         <v>13</v>
       </c>
-      <c r="E33" s="1">
-        <v>7</v>
-      </c>
-      <c r="F33" s="1">
-        <v>4</v>
-      </c>
       <c r="G33" s="1">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="H33" s="1">
-        <v>113</v>
+        <v>219</v>
       </c>
       <c r="I33" s="1">
-        <v>96</v>
+        <v>225</v>
       </c>
       <c r="J33" s="1">
-        <v>17</v>
+        <v>-6</v>
       </c>
       <c r="K33" s="2">
-        <v>0.63600000000000001</v>
+        <v>0.40899999999999997</v>
       </c>
       <c r="L33" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M33" s="1">
         <v>1</v>
       </c>
       <c r="N33" s="1">
-        <v>2</v>
-      </c>
-      <c r="O33" s="11">
+        <v>3</v>
+      </c>
+      <c r="O33" s="13">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
@@ -2989,101 +3053,106 @@
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D34" s="1">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E34" s="1">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F34" s="1">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G34" s="1">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="H34" s="1">
-        <v>109</v>
+        <v>235</v>
       </c>
       <c r="I34" s="1">
-        <v>100</v>
+        <v>227</v>
       </c>
       <c r="J34" s="1">
-        <v>9</v>
-      </c>
-      <c r="K34" s="2">
-        <v>0.54500000000000004</v>
+        <v>8</v>
+      </c>
+      <c r="K34" s="3">
+        <v>0.5</v>
       </c>
       <c r="L34" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M34" s="1">
         <v>0</v>
       </c>
       <c r="N34" s="1">
-        <v>4</v>
-      </c>
-      <c r="O34" s="11">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="P34" s="1"/>
-      <c r="Q34" s="4"/>
+        <v>6</v>
+      </c>
+      <c r="O34" s="13">
+        <f t="shared" si="0"/>
+        <v>10.5</v>
+      </c>
+      <c r="P34" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="R34" s="1"/>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D35" s="1">
+        <v>21</v>
+      </c>
+      <c r="E35" s="1">
         <v>11</v>
       </c>
-      <c r="E35" s="1">
-        <v>6</v>
-      </c>
       <c r="F35" s="1">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G35" s="1">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="H35" s="1">
-        <v>104</v>
+        <v>215</v>
       </c>
       <c r="I35" s="1">
-        <v>110</v>
+        <v>212</v>
       </c>
       <c r="J35" s="1">
-        <v>-6</v>
-      </c>
-      <c r="K35" s="2">
-        <v>0.54500000000000004</v>
+        <v>3</v>
+      </c>
+      <c r="K35" s="3">
+        <v>0.5</v>
       </c>
       <c r="L35" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M35" s="1">
         <v>0</v>
       </c>
       <c r="N35" s="1">
-        <v>5</v>
-      </c>
-      <c r="O35" s="11">
-        <f t="shared" si="0"/>
-        <v>11</v>
+        <v>4</v>
+      </c>
+      <c r="O35" s="13">
+        <f t="shared" si="0"/>
+        <v>10.5</v>
       </c>
       <c r="P35" s="1"/>
       <c r="Q35" s="4"/>
@@ -3091,50 +3160,50 @@
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D36" s="1">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E36" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F36" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G36" s="1">
         <v>11</v>
       </c>
       <c r="H36" s="1">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="I36" s="1">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="J36" s="1">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="K36" s="2">
-        <v>0.45500000000000002</v>
+        <v>0.72699999999999998</v>
       </c>
       <c r="L36" s="1">
         <v>1</v>
       </c>
       <c r="M36" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N36" s="1">
-        <v>6</v>
-      </c>
-      <c r="O36" s="11">
-        <f t="shared" si="0"/>
-        <v>11</v>
+        <v>2</v>
+      </c>
+      <c r="O36" s="13">
+        <f t="shared" si="0"/>
+        <v>21</v>
       </c>
       <c r="P36" s="1"/>
       <c r="Q36" s="4"/>
@@ -3142,50 +3211,50 @@
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D37" s="1">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E37" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F37" s="1">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G37" s="1">
         <v>11</v>
       </c>
       <c r="H37" s="1">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="I37" s="1">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="J37" s="1">
-        <v>-19</v>
+        <v>15</v>
       </c>
       <c r="K37" s="2">
-        <v>0.45500000000000002</v>
+        <v>0.72699999999999998</v>
       </c>
       <c r="L37" s="1">
         <v>1</v>
       </c>
       <c r="M37" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N37" s="1">
-        <v>8</v>
-      </c>
-      <c r="O37" s="11">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <v>2</v>
+      </c>
+      <c r="O37" s="13">
+        <f t="shared" si="0"/>
+        <v>21</v>
       </c>
       <c r="P37" s="1"/>
       <c r="Q37" s="4"/>
@@ -3196,47 +3265,47 @@
         <v>36</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D38" s="1">
+        <v>20</v>
+      </c>
+      <c r="E38" s="1">
+        <v>7</v>
+      </c>
+      <c r="F38" s="1">
+        <v>3</v>
+      </c>
+      <c r="G38" s="1">
         <v>10</v>
       </c>
-      <c r="E38" s="1">
-        <v>5</v>
-      </c>
-      <c r="F38" s="1">
-        <v>6</v>
-      </c>
-      <c r="G38" s="1">
-        <v>11</v>
-      </c>
       <c r="H38" s="1">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I38" s="1">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="J38" s="1">
-        <v>-5</v>
-      </c>
-      <c r="K38" s="2">
-        <v>0.45500000000000002</v>
+        <v>21</v>
+      </c>
+      <c r="K38" s="3">
+        <v>0.7</v>
       </c>
       <c r="L38" s="1">
         <v>1</v>
       </c>
       <c r="M38" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N38" s="1">
-        <v>7</v>
-      </c>
-      <c r="O38" s="11">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <v>3</v>
+      </c>
+      <c r="O38" s="13">
+        <f t="shared" si="0"/>
+        <v>20</v>
       </c>
       <c r="P38" s="1"/>
       <c r="Q38" s="4"/>
@@ -3244,50 +3313,50 @@
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D39" s="1">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E39" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F39" s="1">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G39" s="1">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="H39" s="1">
-        <v>96</v>
+        <v>209</v>
       </c>
       <c r="I39" s="1">
-        <v>105</v>
+        <v>232</v>
       </c>
       <c r="J39" s="1">
-        <v>-9</v>
+        <v>-23</v>
       </c>
       <c r="K39" s="2">
-        <v>0.45500000000000002</v>
+        <v>0.27300000000000002</v>
       </c>
       <c r="L39" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M39" s="1">
         <v>0</v>
       </c>
       <c r="N39" s="1">
-        <v>8</v>
-      </c>
-      <c r="O39" s="11">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <v>9</v>
+      </c>
+      <c r="O39" s="13">
+        <f t="shared" si="0"/>
+        <v>8.5</v>
       </c>
       <c r="P39" s="1"/>
       <c r="Q39" s="4"/>
@@ -3295,37 +3364,37 @@
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D40" s="1">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E40" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F40" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G40" s="1">
         <v>11</v>
       </c>
       <c r="H40" s="1">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I40" s="1">
-        <v>118</v>
+        <v>82</v>
       </c>
       <c r="J40" s="1">
-        <v>-11</v>
+        <v>28</v>
       </c>
       <c r="K40" s="2">
-        <v>0.27300000000000002</v>
+        <v>0.54500000000000004</v>
       </c>
       <c r="L40" s="1">
         <v>1</v>
@@ -3334,11 +3403,11 @@
         <v>0</v>
       </c>
       <c r="N40" s="1">
-        <v>12</v>
-      </c>
-      <c r="O40" s="11">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <v>6</v>
+      </c>
+      <c r="O40" s="13">
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
       <c r="P40" s="1"/>
       <c r="Q40" s="4"/>
@@ -3349,34 +3418,34 @@
         <v>39</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D41" s="1">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E41" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F41" s="1">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G41" s="1">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H41" s="1">
-        <v>23</v>
+        <v>113</v>
       </c>
       <c r="I41" s="1">
-        <v>22</v>
+        <v>114</v>
       </c>
       <c r="J41" s="1">
-        <v>1</v>
-      </c>
-      <c r="K41" s="3">
-        <v>0.5</v>
+        <v>-1</v>
+      </c>
+      <c r="K41" s="2">
+        <v>0.45500000000000002</v>
       </c>
       <c r="L41" s="1">
         <v>1</v>
@@ -3385,15 +3454,780 @@
         <v>0</v>
       </c>
       <c r="N41" s="1">
-        <v>12</v>
-      </c>
-      <c r="O41" s="11">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <v>8</v>
+      </c>
+      <c r="O41" s="13">
+        <f t="shared" si="0"/>
+        <v>16</v>
       </c>
       <c r="P41" s="1"/>
       <c r="Q41" s="4"/>
       <c r="R41" s="1"/>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>39</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D42" s="1">
+        <v>16</v>
+      </c>
+      <c r="E42" s="1">
+        <v>3</v>
+      </c>
+      <c r="F42" s="1">
+        <v>7</v>
+      </c>
+      <c r="G42" s="1">
+        <v>10</v>
+      </c>
+      <c r="H42" s="1">
+        <v>93</v>
+      </c>
+      <c r="I42" s="1">
+        <v>104</v>
+      </c>
+      <c r="J42" s="1">
+        <v>-11</v>
+      </c>
+      <c r="K42" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="L42" s="1">
+        <v>1</v>
+      </c>
+      <c r="M42" s="1">
+        <v>0</v>
+      </c>
+      <c r="N42" s="1">
+        <v>9</v>
+      </c>
+      <c r="O42" s="13">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="P42" s="1"/>
+      <c r="Q42" s="4"/>
+      <c r="R42" s="1"/>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>41</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" s="1">
+        <v>14</v>
+      </c>
+      <c r="E43" s="1">
+        <v>9</v>
+      </c>
+      <c r="F43" s="1">
+        <v>2</v>
+      </c>
+      <c r="G43" s="1">
+        <v>11</v>
+      </c>
+      <c r="H43" s="1">
+        <v>118</v>
+      </c>
+      <c r="I43" s="1">
+        <v>87</v>
+      </c>
+      <c r="J43" s="1">
+        <v>31</v>
+      </c>
+      <c r="K43" s="2">
+        <v>0.81799999999999995</v>
+      </c>
+      <c r="L43" s="1">
+        <v>1</v>
+      </c>
+      <c r="M43" s="1">
+        <v>1</v>
+      </c>
+      <c r="N43" s="1">
+        <v>1</v>
+      </c>
+      <c r="O43" s="13">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="P43" s="1"/>
+      <c r="Q43" s="4"/>
+      <c r="R43" s="1"/>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>42</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" s="1">
+        <v>13</v>
+      </c>
+      <c r="E44" s="1">
+        <v>7</v>
+      </c>
+      <c r="F44" s="1">
+        <v>4</v>
+      </c>
+      <c r="G44" s="1">
+        <v>11</v>
+      </c>
+      <c r="H44" s="1">
+        <v>113</v>
+      </c>
+      <c r="I44" s="1">
+        <v>96</v>
+      </c>
+      <c r="J44" s="1">
+        <v>17</v>
+      </c>
+      <c r="K44" s="2">
+        <v>0.63600000000000001</v>
+      </c>
+      <c r="L44" s="1">
+        <v>1</v>
+      </c>
+      <c r="M44" s="1">
+        <v>1</v>
+      </c>
+      <c r="N44" s="1">
+        <v>2</v>
+      </c>
+      <c r="O44" s="13">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="P44" s="1"/>
+      <c r="Q44" s="4"/>
+      <c r="R44" s="1"/>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>43</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D45" s="1">
+        <v>12</v>
+      </c>
+      <c r="E45" s="1">
+        <v>7</v>
+      </c>
+      <c r="F45" s="1">
+        <v>4</v>
+      </c>
+      <c r="G45" s="1">
+        <v>11</v>
+      </c>
+      <c r="H45" s="1">
+        <v>118</v>
+      </c>
+      <c r="I45" s="1">
+        <v>98</v>
+      </c>
+      <c r="J45" s="1">
+        <v>20</v>
+      </c>
+      <c r="K45" s="2">
+        <v>0.63600000000000001</v>
+      </c>
+      <c r="L45" s="1">
+        <v>1</v>
+      </c>
+      <c r="M45" s="1">
+        <v>1</v>
+      </c>
+      <c r="N45" s="1">
+        <v>3</v>
+      </c>
+      <c r="O45" s="13">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="P45" s="1"/>
+      <c r="Q45" s="4"/>
+      <c r="R45" s="1"/>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>43</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" s="1">
+        <v>12</v>
+      </c>
+      <c r="E46" s="1">
+        <v>6</v>
+      </c>
+      <c r="F46" s="1">
+        <v>5</v>
+      </c>
+      <c r="G46" s="1">
+        <v>11</v>
+      </c>
+      <c r="H46" s="1">
+        <v>109</v>
+      </c>
+      <c r="I46" s="1">
+        <v>100</v>
+      </c>
+      <c r="J46" s="1">
+        <v>9</v>
+      </c>
+      <c r="K46" s="2">
+        <v>0.54500000000000004</v>
+      </c>
+      <c r="L46" s="1">
+        <v>1</v>
+      </c>
+      <c r="M46" s="1">
+        <v>0</v>
+      </c>
+      <c r="N46" s="1">
+        <v>4</v>
+      </c>
+      <c r="O46" s="13">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="P46" s="1"/>
+      <c r="Q46" s="4"/>
+      <c r="R46" s="1"/>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>43</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D47" s="1">
+        <v>12</v>
+      </c>
+      <c r="E47" s="1">
+        <v>6</v>
+      </c>
+      <c r="F47" s="1">
+        <v>5</v>
+      </c>
+      <c r="G47" s="1">
+        <v>11</v>
+      </c>
+      <c r="H47" s="1">
+        <v>109</v>
+      </c>
+      <c r="I47" s="1">
+        <v>100</v>
+      </c>
+      <c r="J47" s="1">
+        <v>9</v>
+      </c>
+      <c r="K47" s="2">
+        <v>0.54500000000000004</v>
+      </c>
+      <c r="L47" s="1">
+        <v>1</v>
+      </c>
+      <c r="M47" s="1">
+        <v>0</v>
+      </c>
+      <c r="N47" s="1">
+        <v>4</v>
+      </c>
+      <c r="O47" s="13">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="P47" s="1"/>
+      <c r="Q47" s="4"/>
+      <c r="R47" s="1"/>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>46</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D48" s="1">
+        <v>11</v>
+      </c>
+      <c r="E48" s="1">
+        <v>6</v>
+      </c>
+      <c r="F48" s="1">
+        <v>5</v>
+      </c>
+      <c r="G48" s="1">
+        <v>11</v>
+      </c>
+      <c r="H48" s="1">
+        <v>104</v>
+      </c>
+      <c r="I48" s="1">
+        <v>110</v>
+      </c>
+      <c r="J48" s="1">
+        <v>-6</v>
+      </c>
+      <c r="K48" s="2">
+        <v>0.54500000000000004</v>
+      </c>
+      <c r="L48" s="1">
+        <v>1</v>
+      </c>
+      <c r="M48" s="1">
+        <v>0</v>
+      </c>
+      <c r="N48" s="1">
+        <v>5</v>
+      </c>
+      <c r="O48" s="13">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="P48" s="1"/>
+      <c r="Q48" s="4"/>
+      <c r="R48" s="1"/>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>47</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D49" s="1">
+        <v>10</v>
+      </c>
+      <c r="E49" s="1">
+        <v>5</v>
+      </c>
+      <c r="F49" s="1">
+        <v>6</v>
+      </c>
+      <c r="G49" s="1">
+        <v>11</v>
+      </c>
+      <c r="H49" s="1">
+        <v>110</v>
+      </c>
+      <c r="I49" s="1">
+        <v>115</v>
+      </c>
+      <c r="J49" s="1">
+        <v>-5</v>
+      </c>
+      <c r="K49" s="2">
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="L49" s="1">
+        <v>1</v>
+      </c>
+      <c r="M49" s="1">
+        <v>0</v>
+      </c>
+      <c r="N49" s="1">
+        <v>7</v>
+      </c>
+      <c r="O49" s="13">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="P49" s="1"/>
+      <c r="Q49" s="4"/>
+      <c r="R49" s="1"/>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>47</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D50" s="1">
+        <v>10</v>
+      </c>
+      <c r="E50" s="1">
+        <v>6</v>
+      </c>
+      <c r="F50" s="1">
+        <v>5</v>
+      </c>
+      <c r="G50" s="1">
+        <v>11</v>
+      </c>
+      <c r="H50" s="1">
+        <v>113</v>
+      </c>
+      <c r="I50" s="1">
+        <v>111</v>
+      </c>
+      <c r="J50" s="1">
+        <v>2</v>
+      </c>
+      <c r="K50" s="2">
+        <v>0.54500000000000004</v>
+      </c>
+      <c r="L50" s="1">
+        <v>1</v>
+      </c>
+      <c r="M50" s="1">
+        <v>0</v>
+      </c>
+      <c r="N50" s="1">
+        <v>7</v>
+      </c>
+      <c r="O50" s="13">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="P50" s="1"/>
+      <c r="Q50" s="4"/>
+      <c r="R50" s="1"/>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>47</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D51" s="1">
+        <v>10</v>
+      </c>
+      <c r="E51" s="1">
+        <v>5</v>
+      </c>
+      <c r="F51" s="1">
+        <v>6</v>
+      </c>
+      <c r="G51" s="1">
+        <v>11</v>
+      </c>
+      <c r="H51" s="1">
+        <v>95</v>
+      </c>
+      <c r="I51" s="1">
+        <v>114</v>
+      </c>
+      <c r="J51" s="1">
+        <v>-19</v>
+      </c>
+      <c r="K51" s="2">
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="L51" s="1">
+        <v>1</v>
+      </c>
+      <c r="M51" s="1">
+        <v>0</v>
+      </c>
+      <c r="N51" s="1">
+        <v>8</v>
+      </c>
+      <c r="O51" s="13">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="P51" s="1"/>
+      <c r="Q51" s="4"/>
+      <c r="R51" s="1"/>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>47</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D52" s="1">
+        <v>10</v>
+      </c>
+      <c r="E52" s="1">
+        <v>5</v>
+      </c>
+      <c r="F52" s="1">
+        <v>6</v>
+      </c>
+      <c r="G52" s="1">
+        <v>11</v>
+      </c>
+      <c r="H52" s="1">
+        <v>96</v>
+      </c>
+      <c r="I52" s="1">
+        <v>105</v>
+      </c>
+      <c r="J52" s="1">
+        <v>-9</v>
+      </c>
+      <c r="K52" s="2">
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="L52" s="1">
+        <v>1</v>
+      </c>
+      <c r="M52" s="1">
+        <v>0</v>
+      </c>
+      <c r="N52" s="1">
+        <v>8</v>
+      </c>
+      <c r="O52" s="13">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="P52" s="1"/>
+      <c r="Q52" s="4"/>
+      <c r="R52" s="1"/>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>47</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D53" s="1">
+        <v>10</v>
+      </c>
+      <c r="E53" s="1">
+        <v>6</v>
+      </c>
+      <c r="F53" s="1">
+        <v>5</v>
+      </c>
+      <c r="G53" s="1">
+        <v>11</v>
+      </c>
+      <c r="H53" s="1">
+        <v>100</v>
+      </c>
+      <c r="I53" s="1">
+        <v>102</v>
+      </c>
+      <c r="J53" s="1">
+        <v>-2</v>
+      </c>
+      <c r="K53" s="2">
+        <v>0.54500000000000004</v>
+      </c>
+      <c r="L53" s="1">
+        <v>1</v>
+      </c>
+      <c r="M53" s="1">
+        <v>0</v>
+      </c>
+      <c r="N53" s="1">
+        <v>7</v>
+      </c>
+      <c r="O53" s="13">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="P53" s="1"/>
+      <c r="Q53" s="4"/>
+      <c r="R53" s="1"/>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>52</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D54" s="1">
+        <v>9</v>
+      </c>
+      <c r="E54" s="1">
+        <v>3</v>
+      </c>
+      <c r="F54" s="1">
+        <v>8</v>
+      </c>
+      <c r="G54" s="1">
+        <v>11</v>
+      </c>
+      <c r="H54" s="1">
+        <v>79</v>
+      </c>
+      <c r="I54" s="1">
+        <v>113</v>
+      </c>
+      <c r="J54" s="1">
+        <v>-34</v>
+      </c>
+      <c r="K54" s="2">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="L54" s="1">
+        <v>1</v>
+      </c>
+      <c r="M54" s="1">
+        <v>0</v>
+      </c>
+      <c r="N54" s="1">
+        <v>10</v>
+      </c>
+      <c r="O54" s="13">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="P54" s="1"/>
+      <c r="Q54" s="4"/>
+      <c r="R54" s="1"/>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>53</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D55" s="1">
+        <v>8</v>
+      </c>
+      <c r="E55" s="1">
+        <v>3</v>
+      </c>
+      <c r="F55" s="1">
+        <v>8</v>
+      </c>
+      <c r="G55" s="1">
+        <v>11</v>
+      </c>
+      <c r="H55" s="1">
+        <v>107</v>
+      </c>
+      <c r="I55" s="1">
+        <v>118</v>
+      </c>
+      <c r="J55" s="1">
+        <v>-11</v>
+      </c>
+      <c r="K55" s="2">
+        <v>0.27300000000000002</v>
+      </c>
+      <c r="L55" s="1">
+        <v>1</v>
+      </c>
+      <c r="M55" s="1">
+        <v>0</v>
+      </c>
+      <c r="N55" s="1">
+        <v>12</v>
+      </c>
+      <c r="O55" s="13">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="P55" s="1"/>
+      <c r="Q55" s="4"/>
+      <c r="R55" s="1"/>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>53</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D56" s="1">
+        <v>8</v>
+      </c>
+      <c r="E56" s="1">
+        <v>1</v>
+      </c>
+      <c r="F56" s="1">
+        <v>1</v>
+      </c>
+      <c r="G56" s="1">
+        <v>2</v>
+      </c>
+      <c r="H56" s="1">
+        <v>23</v>
+      </c>
+      <c r="I56" s="1">
+        <v>22</v>
+      </c>
+      <c r="J56" s="1">
+        <v>1</v>
+      </c>
+      <c r="K56" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="L56" s="1">
+        <v>1</v>
+      </c>
+      <c r="M56" s="1">
+        <v>0</v>
+      </c>
+      <c r="N56" s="1">
+        <v>12</v>
+      </c>
+      <c r="O56" s="13">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="P56" s="1"/>
+      <c r="Q56" s="4"/>
+      <c r="R56" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Standings: Dave's new links for Newbridge Wk 9, Carpenters Wk 6, weekly table
Switched the three share ids the 6 AM page watcher flagged on 2026-10-30
(Jay approved). Season ids unchanged. Watcher fixture refreshed to today's page.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/importer/live/standings/Player-Rankings-HnAtFNN1bzW2DuOVGi3K.xlsx
+++ b/importer/live/standings/Player-Rankings-HnAtFNN1bzW2DuOVGi3K.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/E914DC20F5C50B12/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{618426AC-D233-4601-9FC5-EAA5BC0F96D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5038328-4E40-4044-8465-A93FAC8D4825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F00FA0E0-35F8-4997-80F6-A0D8020722AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8BF7D5C3-A8ED-4D57-8D92-2F6C23274EB4}"/>
   </bookViews>
   <sheets>
     <sheet name="Player-Rankings-HnAtFNN1bzW2DuO" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="81">
   <si>
     <t>Rank</t>
   </si>
@@ -43,39 +43,39 @@
     <t>Win %</t>
   </si>
   <si>
+    <t>Josh Judge</t>
+  </si>
+  <si>
+    <t>Merrick in a pickle</t>
+  </si>
+  <si>
     <t>Robert Player</t>
   </si>
   <si>
-    <t>Merrick in a pickle</t>
-  </si>
-  <si>
-    <t>Josh Judge</t>
-  </si>
-  <si>
     <t>Angel V</t>
   </si>
   <si>
     <t>Michael Spezio</t>
   </si>
   <si>
+    <t>Noah Hackmack</t>
+  </si>
+  <si>
     <t>Rex Bunt</t>
   </si>
   <si>
-    <t>Noah Hackmack</t>
-  </si>
-  <si>
     <t>Vincent Cusumano</t>
   </si>
   <si>
+    <t>Jeff Fein</t>
+  </si>
+  <si>
+    <t>Mike Breitinger</t>
+  </si>
+  <si>
     <t>Adam Kalyvas</t>
   </si>
   <si>
-    <t>Jeff Fein</t>
-  </si>
-  <si>
-    <t>Mike Breitinger</t>
-  </si>
-  <si>
     <t>Jeff Hersh</t>
   </si>
   <si>
@@ -91,31 +91,40 @@
     <t>Adam Stork</t>
   </si>
   <si>
+    <t>Stephen Rizzi</t>
+  </si>
+  <si>
+    <t>Chris Paolina</t>
+  </si>
+  <si>
     <t>Peter Prochilo</t>
   </si>
   <si>
     <t>BOX PICKLEBALL</t>
   </si>
   <si>
-    <t>Chris Paolina</t>
-  </si>
-  <si>
-    <t>Stephen Rizzi</t>
-  </si>
-  <si>
     <t>Lauren Glodny</t>
   </si>
   <si>
+    <t>Mark Lazo</t>
+  </si>
+  <si>
+    <t>PxP PC</t>
+  </si>
+  <si>
     <t>Gregg Dickens</t>
   </si>
   <si>
     <t>Nicole Beiner</t>
   </si>
   <si>
-    <t>Mark Lazo</t>
-  </si>
-  <si>
-    <t>PxP PC</t>
+    <t>Bethuel Bayawa</t>
+  </si>
+  <si>
+    <t>Mikel Strauch</t>
+  </si>
+  <si>
+    <t>Eran Dekel</t>
   </si>
   <si>
     <t>Robert Mentz</t>
@@ -127,19 +136,13 @@
     <t>LI-Kick</t>
   </si>
   <si>
-    <t>Bethuel Bayawa</t>
+    <t>Christie Simmons</t>
   </si>
   <si>
     <t>Glenn Saenz</t>
   </si>
   <si>
-    <t>Mikel Strauch</t>
-  </si>
-  <si>
-    <t>Christie Simmons</t>
-  </si>
-  <si>
-    <t>Eran Dekel</t>
+    <t>Kenny Jee</t>
   </si>
   <si>
     <t>Shane Morrison</t>
@@ -154,9 +157,6 @@
     <t>Edward Wahl</t>
   </si>
   <si>
-    <t>Kenny Jee</t>
-  </si>
-  <si>
     <t>Richard Vaselli</t>
   </si>
   <si>
@@ -166,6 +166,9 @@
     <t>Paul Ilan</t>
   </si>
   <si>
+    <t>David Huber</t>
+  </si>
+  <si>
     <t>Olivia O’Keefe</t>
   </si>
   <si>
@@ -196,9 +199,6 @@
     <t>Charles Maione</t>
   </si>
   <si>
-    <t>David Huber</t>
-  </si>
-  <si>
     <t>Alexia Yaziciyan</t>
   </si>
   <si>
@@ -211,6 +211,12 @@
     <t>Lori McBride</t>
   </si>
   <si>
+    <t>Arthur Galo</t>
+  </si>
+  <si>
+    <t>1 Pickleball Plaza</t>
+  </si>
+  <si>
     <t>Michael Scancarello</t>
   </si>
   <si>
@@ -250,10 +256,10 @@
     <t>Gold</t>
   </si>
   <si>
-    <t>NBI WEDNESDAY NIGHT</t>
-  </si>
-  <si>
-    <t>WEEK 8</t>
+    <t>NBI BIG DOGS</t>
+  </si>
+  <si>
+    <t>WEEK 9</t>
   </si>
   <si>
     <t>MERRICK IN A PICKLE</t>
@@ -404,17 +410,17 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Georgia Pro Cond Black"/>
-      <family val="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="20"/>
+      <sz val="22"/>
       <color theme="1"/>
-      <name val="Kermit Extrabold"/>
-      <family val="2"/>
+      <name val="ADLaM Display"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -608,19 +614,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.89999084444715716"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
+        <fgColor theme="2" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -801,7 +813,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -812,57 +824,65 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="33" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="36" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="19" fillId="36" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="37" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="19" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="38" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="37" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="18" fillId="37" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="18" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1240,211 +1260,209 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A317B30-3C65-4F10-B586-709463314FD3}">
-  <dimension ref="A1:R56"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F42A5AD-1A24-4B33-9129-1A5E86BE5E88}">
+  <dimension ref="A1:R57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" style="14"/>
-    <col min="17" max="17" width="9.140625" style="5"/>
+    <col min="2" max="3" width="18.28515625" customWidth="1"/>
+    <col min="15" max="15" width="9.140625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="16" customFormat="1" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17"/>
-      <c r="B1" s="17" t="s">
+    <row r="1" spans="1:18" s="22" customFormat="1" ht="30" x14ac:dyDescent="0.5">
+      <c r="A1" s="23"/>
+      <c r="B1" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="O1" s="24"/>
+      <c r="P1" s="23"/>
+      <c r="Q1" s="23"/>
+      <c r="R1" s="23"/>
+    </row>
+    <row r="2" spans="1:18" s="21" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="I2" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="K2" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="L2" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="M2" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="N2" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="O2" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="P2" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q2" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17" t="s">
+      <c r="R2" s="25" t="s">
         <v>77</v>
-      </c>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="O1" s="18"/>
-      <c r="P1" s="17"/>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="17"/>
-    </row>
-    <row r="2" spans="1:18" s="15" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="20" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="20" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="H2" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="I2" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="J2" s="20" t="s">
-        <v>68</v>
-      </c>
-      <c r="K2" s="20" t="s">
-        <v>6</v>
-      </c>
-      <c r="L2" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="M2" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="N2" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="O2" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="P2" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q2" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="R2" s="20" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="15" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="6">
-        <v>167</v>
-      </c>
-      <c r="E3" s="6">
-        <v>54</v>
+      <c r="D3" s="4">
+        <v>175</v>
+      </c>
+      <c r="E3" s="4">
+        <v>59</v>
       </c>
       <c r="F3" s="1">
-        <v>33</v>
-      </c>
-      <c r="G3" s="9">
+        <v>28</v>
+      </c>
+      <c r="G3" s="1">
         <v>87</v>
       </c>
-      <c r="H3" s="6">
-        <v>934</v>
+      <c r="H3" s="1">
+        <v>915</v>
       </c>
       <c r="I3" s="1">
-        <v>828</v>
-      </c>
-      <c r="J3" s="6">
-        <v>106</v>
-      </c>
-      <c r="K3" s="2">
-        <v>0.621</v>
-      </c>
-      <c r="L3" s="6">
-        <v>8</v>
-      </c>
-      <c r="M3" s="6">
-        <v>5</v>
+        <v>822</v>
+      </c>
+      <c r="J3" s="19">
+        <v>93</v>
+      </c>
+      <c r="K3" s="11">
+        <v>0.67800000000000005</v>
+      </c>
+      <c r="L3" s="1">
+        <v>8</v>
+      </c>
+      <c r="M3" s="4">
+        <v>6</v>
       </c>
       <c r="N3" s="1">
         <v>1</v>
       </c>
-      <c r="O3" s="13">
+      <c r="O3" s="10">
         <f>D3/L3</f>
-        <v>20.875</v>
-      </c>
-      <c r="P3" s="6">
-        <v>8</v>
-      </c>
-      <c r="Q3" s="8">
+        <v>21.875</v>
+      </c>
+      <c r="P3" s="4">
+        <v>8</v>
+      </c>
+      <c r="Q3" s="7">
         <f>P3/L3</f>
         <v>1</v>
       </c>
-      <c r="R3" s="6">
-        <v>3</v>
+      <c r="R3" s="4">
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="16" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="9">
-        <v>150</v>
-      </c>
-      <c r="E4" s="9">
-        <v>50</v>
+      <c r="D4" s="13">
+        <v>167</v>
+      </c>
+      <c r="E4" s="17">
+        <v>54</v>
       </c>
       <c r="F4" s="1">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G4" s="1">
-        <v>76</v>
-      </c>
-      <c r="H4" s="1">
-        <v>794</v>
+        <v>87</v>
+      </c>
+      <c r="H4" s="17">
+        <v>934</v>
       </c>
       <c r="I4" s="1">
-        <v>728</v>
-      </c>
-      <c r="J4" s="1">
-        <v>66</v>
-      </c>
-      <c r="K4" s="10">
-        <v>0.65800000000000003</v>
+        <v>828</v>
+      </c>
+      <c r="J4" s="13">
+        <v>106</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0.621</v>
       </c>
       <c r="L4" s="1">
-        <v>7</v>
-      </c>
-      <c r="M4" s="6">
+        <v>8</v>
+      </c>
+      <c r="M4" s="13">
         <v>5</v>
       </c>
       <c r="N4" s="1">
         <v>1</v>
       </c>
-      <c r="O4" s="13">
-        <f t="shared" ref="O4:O56" si="0">D4/L4</f>
-        <v>21.428571428571427</v>
-      </c>
-      <c r="P4" s="1">
-        <v>7</v>
-      </c>
-      <c r="Q4" s="8">
-        <f t="shared" ref="Q4:Q34" si="1">P4/L4</f>
-        <v>1</v>
-      </c>
-      <c r="R4" s="6">
+      <c r="O4" s="14">
+        <f t="shared" ref="O4:O57" si="0">D4/L4</f>
+        <v>20.875</v>
+      </c>
+      <c r="P4" s="4">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="7">
+        <f t="shared" ref="Q4:Q35" si="1">P4/L4</f>
+        <v>1</v>
+      </c>
+      <c r="R4" s="13">
         <v>3</v>
       </c>
     </row>
@@ -1452,96 +1470,96 @@
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="18" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="11">
-        <v>140</v>
-      </c>
-      <c r="E5" s="11">
-        <v>49</v>
+      <c r="D5" s="19">
+        <v>161</v>
+      </c>
+      <c r="E5" s="13">
+        <v>58</v>
       </c>
       <c r="F5" s="1">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G5" s="1">
-        <v>77</v>
-      </c>
-      <c r="H5" s="1">
-        <v>828</v>
+        <v>88</v>
+      </c>
+      <c r="H5" s="13">
+        <v>949</v>
       </c>
       <c r="I5" s="1">
-        <v>758</v>
-      </c>
-      <c r="J5" s="11">
-        <v>70</v>
-      </c>
-      <c r="K5" s="12">
-        <v>0.63600000000000001</v>
+        <v>856</v>
+      </c>
+      <c r="J5" s="1">
+        <v>93</v>
+      </c>
+      <c r="K5" s="2">
+        <v>0.65900000000000003</v>
       </c>
       <c r="L5" s="1">
-        <v>7</v>
-      </c>
-      <c r="M5" s="11">
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="M5" s="13">
+        <v>5</v>
       </c>
       <c r="N5" s="1">
         <v>1</v>
       </c>
-      <c r="O5" s="13">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="P5" s="1">
-        <v>7</v>
-      </c>
-      <c r="Q5" s="8">
+      <c r="O5" s="20">
+        <f t="shared" si="0"/>
+        <v>20.125</v>
+      </c>
+      <c r="P5" s="4">
+        <v>8</v>
+      </c>
+      <c r="Q5" s="7">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="R5" s="11">
-        <v>2</v>
+      <c r="R5" s="19">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="1">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="E6" s="1">
+        <v>46</v>
+      </c>
+      <c r="F6" s="1">
         <v>41</v>
       </c>
-      <c r="F6" s="1">
-        <v>35</v>
-      </c>
       <c r="G6" s="1">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="H6" s="1">
-        <v>742</v>
+        <v>846</v>
       </c>
       <c r="I6" s="1">
-        <v>756</v>
+        <v>868</v>
       </c>
       <c r="J6" s="1">
-        <v>-14</v>
+        <v>-22</v>
       </c>
       <c r="K6" s="2">
-        <v>0.53900000000000003</v>
+        <v>0.52900000000000003</v>
       </c>
       <c r="L6" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M6" s="1">
         <v>2</v>
@@ -1549,16 +1567,16 @@
       <c r="N6" s="1">
         <v>2</v>
       </c>
-      <c r="O6" s="13">
-        <f t="shared" si="0"/>
-        <v>17.571428571428573</v>
+      <c r="O6" s="8">
+        <f t="shared" si="0"/>
+        <v>17.5</v>
       </c>
       <c r="P6" s="1">
         <v>7</v>
       </c>
-      <c r="Q6" s="8">
+      <c r="Q6" s="6">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.875</v>
       </c>
       <c r="R6" s="1"/>
     </row>
@@ -1566,57 +1584,57 @@
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="1">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="E7" s="1">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="F7" s="1">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="G7" s="1">
-        <v>85</v>
-      </c>
-      <c r="H7" s="11">
-        <v>854</v>
+        <v>77</v>
+      </c>
+      <c r="H7" s="1">
+        <v>791</v>
       </c>
       <c r="I7" s="1">
-        <v>832</v>
-      </c>
-      <c r="J7" s="1">
-        <v>22</v>
-      </c>
-      <c r="K7" s="2">
-        <v>0.52900000000000003</v>
-      </c>
-      <c r="L7" s="6">
-        <v>8</v>
+        <v>676</v>
+      </c>
+      <c r="J7" s="4">
+        <v>115</v>
+      </c>
+      <c r="K7" s="12">
+        <v>0.66200000000000003</v>
+      </c>
+      <c r="L7" s="1">
+        <v>7</v>
       </c>
       <c r="M7" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N7" s="1">
         <v>1</v>
       </c>
-      <c r="O7" s="13">
-        <f t="shared" si="0"/>
-        <v>15.25</v>
+      <c r="O7" s="8">
+        <f t="shared" si="0"/>
+        <v>19.857142857142858</v>
       </c>
       <c r="P7" s="1">
         <v>6</v>
       </c>
-      <c r="Q7" s="4">
+      <c r="Q7" s="6">
         <f t="shared" si="1"/>
-        <v>0.75</v>
-      </c>
-      <c r="R7" s="1">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="R7" s="19">
         <v>1</v>
       </c>
     </row>
@@ -1624,38 +1642,38 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="1">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="E8" s="1">
+        <v>52</v>
+      </c>
+      <c r="F8" s="1">
         <v>44</v>
       </c>
-      <c r="F8" s="1">
-        <v>22</v>
-      </c>
-      <c r="G8" s="1">
-        <v>66</v>
-      </c>
-      <c r="H8" s="1">
-        <v>681</v>
+      <c r="G8" s="13">
+        <v>96</v>
+      </c>
+      <c r="H8" s="4">
+        <v>962</v>
       </c>
       <c r="I8" s="1">
-        <v>578</v>
-      </c>
-      <c r="J8" s="9">
-        <v>103</v>
-      </c>
-      <c r="K8" s="7">
-        <v>0.66700000000000004</v>
-      </c>
-      <c r="L8" s="1">
-        <v>6</v>
+        <v>928</v>
+      </c>
+      <c r="J8" s="1">
+        <v>34</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0.54200000000000004</v>
+      </c>
+      <c r="L8" s="4">
+        <v>9</v>
       </c>
       <c r="M8" s="1">
         <v>3</v>
@@ -1663,18 +1681,18 @@
       <c r="N8" s="1">
         <v>1</v>
       </c>
-      <c r="O8" s="13">
-        <f t="shared" si="0"/>
-        <v>20</v>
+      <c r="O8" s="8">
+        <f t="shared" si="0"/>
+        <v>15</v>
       </c>
       <c r="P8" s="1">
         <v>6</v>
       </c>
-      <c r="Q8" s="8">
+      <c r="Q8" s="6">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="R8" s="1">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="R8" s="19">
         <v>1</v>
       </c>
     </row>
@@ -1682,38 +1700,38 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="1">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="E9" s="1">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F9" s="1">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G9" s="1">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="H9" s="1">
-        <v>762</v>
+        <v>863</v>
       </c>
       <c r="I9" s="1">
-        <v>772</v>
+        <v>892</v>
       </c>
       <c r="J9" s="1">
-        <v>-10</v>
-      </c>
-      <c r="K9" s="3">
-        <v>0.5</v>
+        <v>-29</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0.48299999999999998</v>
       </c>
       <c r="L9" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M9" s="1">
         <v>0</v>
@@ -1721,16 +1739,16 @@
       <c r="N9" s="1">
         <v>4</v>
       </c>
-      <c r="O9" s="13">
-        <f t="shared" si="0"/>
-        <v>16.428571428571427</v>
+      <c r="O9" s="8">
+        <f t="shared" si="0"/>
+        <v>16.375</v>
       </c>
       <c r="P9" s="1">
-        <v>6</v>
-      </c>
-      <c r="Q9" s="4">
+        <v>7</v>
+      </c>
+      <c r="Q9" s="6">
         <f t="shared" si="1"/>
-        <v>0.8571428571428571</v>
+        <v>0.875</v>
       </c>
       <c r="R9" s="1"/>
     </row>
@@ -1738,55 +1756,55 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="1">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="E10" s="1">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="F10" s="1">
-        <v>41</v>
-      </c>
-      <c r="G10" s="9">
-        <v>87</v>
-      </c>
-      <c r="H10" s="9">
-        <v>866</v>
+        <v>48</v>
+      </c>
+      <c r="G10" s="1">
+        <v>89</v>
+      </c>
+      <c r="H10" s="1">
+        <v>854</v>
       </c>
       <c r="I10" s="1">
-        <v>842</v>
+        <v>889</v>
       </c>
       <c r="J10" s="1">
-        <v>24</v>
+        <v>-35</v>
       </c>
       <c r="K10" s="2">
-        <v>0.52900000000000003</v>
-      </c>
-      <c r="L10" s="6">
+        <v>0.46100000000000002</v>
+      </c>
+      <c r="L10" s="1">
         <v>8</v>
       </c>
       <c r="M10" s="1">
+        <v>1</v>
+      </c>
+      <c r="N10" s="1">
         <v>3</v>
       </c>
-      <c r="N10" s="1">
-        <v>2</v>
-      </c>
-      <c r="O10" s="13">
-        <f t="shared" si="0"/>
-        <v>13.625</v>
+      <c r="O10" s="8">
+        <f t="shared" si="0"/>
+        <v>14.75</v>
       </c>
       <c r="P10" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q10" s="4">
+        <v>6</v>
+      </c>
+      <c r="Q10" s="6">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="R10" s="1"/>
     </row>
@@ -1794,55 +1812,55 @@
       <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="1">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="E11" s="1">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F11" s="1">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G11" s="1">
         <v>77</v>
       </c>
       <c r="H11" s="1">
-        <v>743</v>
+        <v>777</v>
       </c>
       <c r="I11" s="1">
-        <v>772</v>
+        <v>781</v>
       </c>
       <c r="J11" s="1">
-        <v>-29</v>
+        <v>-4</v>
       </c>
       <c r="K11" s="2">
-        <v>0.45500000000000002</v>
+        <v>0.48099999999999998</v>
       </c>
       <c r="L11" s="1">
         <v>7</v>
       </c>
       <c r="M11" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N11" s="1">
-        <v>3</v>
-      </c>
-      <c r="O11" s="13">
-        <f t="shared" si="0"/>
-        <v>15.285714285714286</v>
+        <v>5</v>
+      </c>
+      <c r="O11" s="8">
+        <f t="shared" si="0"/>
+        <v>16.714285714285715</v>
       </c>
       <c r="P11" s="1">
-        <v>6</v>
-      </c>
-      <c r="Q11" s="4">
+        <v>7</v>
+      </c>
+      <c r="Q11" s="7">
         <f t="shared" si="1"/>
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
       <c r="R11" s="1"/>
     </row>
@@ -1850,55 +1868,55 @@
       <c r="A12" s="1">
         <v>10</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="1">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="E12" s="1">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="F12" s="1">
-        <v>32</v>
-      </c>
-      <c r="G12" s="1">
-        <v>66</v>
+        <v>42</v>
+      </c>
+      <c r="G12" s="17">
+        <v>90</v>
       </c>
       <c r="H12" s="1">
-        <v>682</v>
+        <v>897</v>
       </c>
       <c r="I12" s="1">
-        <v>669</v>
+        <v>869</v>
       </c>
       <c r="J12" s="1">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="K12" s="2">
-        <v>0.51500000000000001</v>
-      </c>
-      <c r="L12" s="1">
-        <v>6</v>
+        <v>0.53300000000000003</v>
+      </c>
+      <c r="L12" s="4">
+        <v>9</v>
       </c>
       <c r="M12" s="1">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N12" s="1">
-        <v>5</v>
-      </c>
-      <c r="O12" s="13">
-        <f t="shared" si="0"/>
-        <v>17</v>
+        <v>2</v>
+      </c>
+      <c r="O12" s="8">
+        <f t="shared" si="0"/>
+        <v>12.888888888888889</v>
       </c>
       <c r="P12" s="1">
-        <v>6</v>
-      </c>
-      <c r="Q12" s="4">
+        <v>4</v>
+      </c>
+      <c r="Q12" s="6">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.44444444444444442</v>
       </c>
       <c r="R12" s="1"/>
     </row>
@@ -1945,17 +1963,12 @@
       <c r="N13" s="1">
         <v>1</v>
       </c>
-      <c r="O13" s="13">
+      <c r="O13" s="8">
         <f t="shared" si="0"/>
         <v>14.428571428571429</v>
       </c>
-      <c r="P13" s="1">
-        <v>6</v>
-      </c>
-      <c r="Q13" s="4">
-        <f t="shared" si="1"/>
-        <v>0.8571428571428571</v>
-      </c>
+      <c r="P13" s="1"/>
+      <c r="Q13" s="6"/>
       <c r="R13" s="1">
         <v>0.5</v>
       </c>
@@ -1964,7 +1977,7 @@
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -1979,7 +1992,7 @@
       <c r="F14" s="1">
         <v>49</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="1">
         <v>88</v>
       </c>
       <c r="H14" s="1">
@@ -1994,7 +2007,7 @@
       <c r="K14" s="2">
         <v>0.443</v>
       </c>
-      <c r="L14" s="6">
+      <c r="L14" s="1">
         <v>8</v>
       </c>
       <c r="M14" s="1">
@@ -2003,14 +2016,14 @@
       <c r="N14" s="1">
         <v>1</v>
       </c>
-      <c r="O14" s="13">
+      <c r="O14" s="8">
         <f t="shared" si="0"/>
         <v>12.5</v>
       </c>
       <c r="P14" s="1">
         <v>4</v>
       </c>
-      <c r="Q14" s="4">
+      <c r="Q14" s="6">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
@@ -2022,38 +2035,38 @@
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="1">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="E15" s="1">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F15" s="1">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="G15" s="1">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="H15" s="1">
-        <v>638</v>
+        <v>733</v>
       </c>
       <c r="I15" s="1">
-        <v>645</v>
+        <v>735</v>
       </c>
       <c r="J15" s="1">
-        <v>-7</v>
+        <v>-2</v>
       </c>
       <c r="K15" s="2">
         <v>0.45500000000000002</v>
       </c>
       <c r="L15" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M15" s="1">
         <v>2</v>
@@ -2061,16 +2074,16 @@
       <c r="N15" s="1">
         <v>3</v>
       </c>
-      <c r="O15" s="13">
-        <f t="shared" si="0"/>
-        <v>14.5</v>
+      <c r="O15" s="8">
+        <f t="shared" si="0"/>
+        <v>14</v>
       </c>
       <c r="P15" s="1">
         <v>4</v>
       </c>
-      <c r="Q15" s="4">
+      <c r="Q15" s="6">
         <f t="shared" si="1"/>
-        <v>0.66666666666666663</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="R15" s="1"/>
     </row>
@@ -2078,38 +2091,38 @@
       <c r="A16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="1">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="E16" s="1">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F16" s="1">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="G16" s="1">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="H16" s="1">
-        <v>614</v>
+        <v>714</v>
       </c>
       <c r="I16" s="1">
-        <v>650</v>
+        <v>762</v>
       </c>
       <c r="J16" s="1">
-        <v>-36</v>
+        <v>-48</v>
       </c>
       <c r="K16" s="2">
-        <v>0.44600000000000001</v>
+        <v>0.434</v>
       </c>
       <c r="L16" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M16" s="1">
         <v>0</v>
@@ -2117,16 +2130,16 @@
       <c r="N16" s="1">
         <v>4</v>
       </c>
-      <c r="O16" s="13">
-        <f t="shared" si="0"/>
-        <v>13.166666666666666</v>
+      <c r="O16" s="8">
+        <f t="shared" si="0"/>
+        <v>12.571428571428571</v>
       </c>
       <c r="P16" s="1">
         <v>4</v>
       </c>
-      <c r="Q16" s="4">
+      <c r="Q16" s="6">
         <f t="shared" si="1"/>
-        <v>0.66666666666666663</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="R16" s="1"/>
     </row>
@@ -2134,55 +2147,55 @@
       <c r="A17" s="1">
         <v>15</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="D17" s="1">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="E17" s="1">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="F17" s="1">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="G17" s="1">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="H17" s="1">
-        <v>531</v>
+        <v>767</v>
       </c>
       <c r="I17" s="1">
-        <v>547</v>
+        <v>748</v>
       </c>
       <c r="J17" s="1">
-        <v>-16</v>
+        <v>19</v>
       </c>
       <c r="K17" s="2">
-        <v>0.436</v>
+        <v>0.48099999999999998</v>
       </c>
       <c r="L17" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M17" s="1">
         <v>0</v>
       </c>
       <c r="N17" s="1">
-        <v>4</v>
-      </c>
-      <c r="O17" s="13">
-        <f t="shared" si="0"/>
-        <v>14.8</v>
+        <v>5</v>
+      </c>
+      <c r="O17" s="8">
+        <f t="shared" si="0"/>
+        <v>12.428571428571429</v>
       </c>
       <c r="P17" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q17" s="4">
+        <v>3</v>
+      </c>
+      <c r="Q17" s="6">
         <f t="shared" si="1"/>
-        <v>0.8</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="R17" s="1"/>
     </row>
@@ -2190,55 +2203,55 @@
       <c r="A18" s="1">
         <v>16</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>25</v>
+      <c r="B18" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="1">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="E18" s="1">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F18" s="1">
-        <v>61</v>
-      </c>
-      <c r="G18" s="9">
-        <v>87</v>
+        <v>65</v>
+      </c>
+      <c r="G18" s="4">
+        <v>97</v>
       </c>
       <c r="H18" s="1">
-        <v>751</v>
+        <v>850</v>
       </c>
       <c r="I18" s="1">
-        <v>922</v>
+        <v>1020</v>
       </c>
       <c r="J18" s="1">
-        <v>-171</v>
-      </c>
-      <c r="K18" s="2">
-        <v>0.29899999999999999</v>
-      </c>
-      <c r="L18" s="6">
-        <v>8</v>
+        <v>-170</v>
+      </c>
+      <c r="K18" s="3">
+        <v>0.33</v>
+      </c>
+      <c r="L18" s="4">
+        <v>9</v>
       </c>
       <c r="M18" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N18" s="1">
-        <v>6</v>
-      </c>
-      <c r="O18" s="13">
-        <f t="shared" si="0"/>
-        <v>8.875</v>
+        <v>3</v>
+      </c>
+      <c r="O18" s="8">
+        <f t="shared" si="0"/>
+        <v>9.2222222222222214</v>
       </c>
       <c r="P18" s="1">
         <v>1</v>
       </c>
-      <c r="Q18" s="4">
+      <c r="Q18" s="6">
         <f t="shared" si="1"/>
-        <v>0.125</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="R18" s="1"/>
     </row>
@@ -2246,35 +2259,35 @@
       <c r="A19" s="1">
         <v>17</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="D19" s="1">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="E19" s="1">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F19" s="1">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G19" s="1">
         <v>66</v>
       </c>
       <c r="H19" s="1">
+        <v>622</v>
+      </c>
+      <c r="I19" s="1">
         <v>655</v>
       </c>
-      <c r="I19" s="1">
-        <v>639</v>
-      </c>
       <c r="J19" s="1">
-        <v>16</v>
-      </c>
-      <c r="K19" s="3">
-        <v>0.47</v>
+        <v>-33</v>
+      </c>
+      <c r="K19" s="2">
+        <v>0.42399999999999999</v>
       </c>
       <c r="L19" s="1">
         <v>6</v>
@@ -2283,18 +2296,18 @@
         <v>0</v>
       </c>
       <c r="N19" s="1">
-        <v>5</v>
-      </c>
-      <c r="O19" s="13">
-        <f t="shared" si="0"/>
-        <v>11.666666666666666</v>
+        <v>4</v>
+      </c>
+      <c r="O19" s="8">
+        <f t="shared" si="0"/>
+        <v>13.666666666666666</v>
       </c>
       <c r="P19" s="1">
-        <v>2</v>
-      </c>
-      <c r="Q19" s="4">
+        <v>4</v>
+      </c>
+      <c r="Q19" s="6">
         <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="R19" s="1"/>
     </row>
@@ -2309,44 +2322,44 @@
         <v>8</v>
       </c>
       <c r="D20" s="1">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="E20" s="1">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="F20" s="1">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="G20" s="1">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="H20" s="1">
-        <v>686</v>
+        <v>794</v>
       </c>
       <c r="I20" s="1">
-        <v>768</v>
+        <v>868</v>
       </c>
       <c r="J20" s="1">
-        <v>-82</v>
+        <v>-74</v>
       </c>
       <c r="K20" s="2">
-        <v>0.39500000000000002</v>
+        <v>0.41399999999999998</v>
       </c>
       <c r="L20" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M20" s="1">
         <v>0</v>
       </c>
       <c r="N20" s="1">
-        <v>5</v>
-      </c>
-      <c r="O20" s="13">
-        <f t="shared" si="0"/>
-        <v>9.8571428571428577</v>
+        <v>4</v>
+      </c>
+      <c r="O20" s="8">
+        <f t="shared" si="0"/>
+        <v>10.125</v>
       </c>
       <c r="P20" s="1"/>
-      <c r="Q20" s="4"/>
+      <c r="Q20" s="6"/>
       <c r="R20" s="1"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
@@ -2357,47 +2370,47 @@
         <v>28</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="D21" s="1">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="E21" s="1">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F21" s="1">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="G21" s="1">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="H21" s="1">
-        <v>325</v>
+        <v>572</v>
       </c>
       <c r="I21" s="1">
-        <v>312</v>
+        <v>544</v>
       </c>
       <c r="J21" s="1">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="K21" s="2">
-        <v>0.53100000000000003</v>
+        <v>0.56399999999999995</v>
       </c>
       <c r="L21" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M21" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N21" s="1">
-        <v>5</v>
-      </c>
-      <c r="O21" s="13">
-        <f t="shared" si="0"/>
-        <v>16.666666666666668</v>
+        <v>2</v>
+      </c>
+      <c r="O21" s="8">
+        <f t="shared" si="0"/>
+        <v>13.4</v>
       </c>
       <c r="P21" s="1"/>
-      <c r="Q21" s="4"/>
+      <c r="Q21" s="6"/>
       <c r="R21" s="1"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
@@ -2405,109 +2418,109 @@
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D22" s="1">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="E22" s="1">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F22" s="1">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="G22" s="1">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="H22" s="1">
-        <v>512</v>
+        <v>436</v>
       </c>
       <c r="I22" s="1">
-        <v>536</v>
+        <v>426</v>
       </c>
       <c r="J22" s="1">
-        <v>-24</v>
+        <v>10</v>
       </c>
       <c r="K22" s="2">
-        <v>0.42599999999999999</v>
+        <v>0.48799999999999999</v>
       </c>
       <c r="L22" s="1">
+        <v>4</v>
+      </c>
+      <c r="M22" s="1">
+        <v>0</v>
+      </c>
+      <c r="N22" s="1">
         <v>5</v>
       </c>
-      <c r="M22" s="1">
-        <v>1</v>
-      </c>
-      <c r="N22" s="1">
-        <v>1</v>
-      </c>
-      <c r="O22" s="13">
-        <f t="shared" si="0"/>
-        <v>9.8000000000000007</v>
-      </c>
-      <c r="P22" s="1">
-        <v>1</v>
-      </c>
-      <c r="Q22" s="4">
-        <f t="shared" si="1"/>
-        <v>0.2</v>
-      </c>
-      <c r="R22" s="1">
-        <v>0.5</v>
-      </c>
+      <c r="O22" s="8">
+        <f t="shared" si="0"/>
+        <v>16.5</v>
+      </c>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="6"/>
+      <c r="R22" s="1"/>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>20</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>30</v>
+        <v>21</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="D23" s="1">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="E23" s="1">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F23" s="1">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G23" s="1">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="H23" s="1">
-        <v>459</v>
+        <v>619</v>
       </c>
       <c r="I23" s="1">
-        <v>434</v>
+        <v>658</v>
       </c>
       <c r="J23" s="1">
-        <v>25</v>
+        <v>-39</v>
       </c>
       <c r="K23" s="2">
-        <v>0.54500000000000004</v>
+        <v>0.38500000000000001</v>
       </c>
       <c r="L23" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M23" s="1">
+        <v>1</v>
+      </c>
+      <c r="N23" s="1">
+        <v>1</v>
+      </c>
+      <c r="O23" s="8">
+        <f t="shared" si="0"/>
+        <v>10.5</v>
+      </c>
+      <c r="P23" s="1">
         <v>2</v>
       </c>
-      <c r="N23" s="1">
-        <v>2</v>
-      </c>
-      <c r="O23" s="13">
-        <f t="shared" si="0"/>
-        <v>12.25</v>
-      </c>
-      <c r="P23" s="1"/>
-      <c r="Q23" s="4"/>
-      <c r="R23" s="1"/>
+      <c r="Q23" s="6">
+        <f t="shared" si="1"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="R23" s="1">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
@@ -2520,63 +2533,60 @@
         <v>8</v>
       </c>
       <c r="D24" s="1">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="E24" s="1">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F24" s="1">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="G24" s="1">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="H24" s="1">
-        <v>452</v>
+        <v>429</v>
       </c>
       <c r="I24" s="1">
-        <v>565</v>
+        <v>409</v>
       </c>
       <c r="J24" s="1">
-        <v>-113</v>
+        <v>20</v>
       </c>
       <c r="K24" s="2">
-        <v>0.25900000000000001</v>
+        <v>0.59099999999999997</v>
       </c>
       <c r="L24" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M24" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N24" s="1">
-        <v>7</v>
-      </c>
-      <c r="O24" s="13">
-        <f t="shared" si="0"/>
-        <v>8.4</v>
-      </c>
-      <c r="P24" s="1">
-        <v>1</v>
-      </c>
-      <c r="Q24" s="4">
-        <f t="shared" si="1"/>
-        <v>0.2</v>
-      </c>
-      <c r="R24" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="O24" s="8">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="6"/>
+      <c r="R24" s="1">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="5" t="s">
         <v>33</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="D25" s="1">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="E25" s="1">
         <v>24</v>
@@ -2588,13 +2598,13 @@
         <v>44</v>
       </c>
       <c r="H25" s="1">
-        <v>440</v>
+        <v>450</v>
       </c>
       <c r="I25" s="1">
-        <v>464</v>
+        <v>425</v>
       </c>
       <c r="J25" s="1">
-        <v>-24</v>
+        <v>25</v>
       </c>
       <c r="K25" s="2">
         <v>0.54500000000000004</v>
@@ -2603,21 +2613,21 @@
         <v>4</v>
       </c>
       <c r="M25" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N25" s="1">
         <v>2</v>
       </c>
-      <c r="O25" s="13">
-        <f t="shared" si="0"/>
-        <v>10.25</v>
+      <c r="O25" s="8">
+        <f t="shared" si="0"/>
+        <v>12.75</v>
       </c>
       <c r="P25" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="4">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="R25" s="1"/>
     </row>
@@ -2625,51 +2635,56 @@
       <c r="A26" s="1">
         <v>24</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>35</v>
+      <c r="B26" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D26" s="1">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="E26" s="1">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F26" s="1">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G26" s="1">
         <v>33</v>
       </c>
       <c r="H26" s="1">
-        <v>333</v>
+        <v>324</v>
       </c>
       <c r="I26" s="1">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="J26" s="1">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="K26" s="2">
-        <v>0.69699999999999995</v>
+        <v>0.57599999999999996</v>
       </c>
       <c r="L26" s="1">
         <v>3</v>
       </c>
       <c r="M26" s="1">
+        <v>1</v>
+      </c>
+      <c r="N26" s="1">
+        <v>1</v>
+      </c>
+      <c r="O26" s="8">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="P26" s="1">
         <v>2</v>
       </c>
-      <c r="N26" s="1">
-        <v>1</v>
-      </c>
-      <c r="O26" s="13">
-        <f t="shared" si="0"/>
-        <v>12.333333333333334</v>
-      </c>
-      <c r="P26" s="1"/>
-      <c r="Q26" s="4"/>
+      <c r="Q26" s="6">
+        <f t="shared" si="1"/>
+        <v>0.66666666666666663</v>
+      </c>
       <c r="R26" s="1">
         <v>0.5</v>
       </c>
@@ -2678,89 +2693,94 @@
       <c r="A27" s="1">
         <v>25</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>36</v>
+      <c r="B27" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D27" s="1">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E27" s="1">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F27" s="1">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="G27" s="1">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="H27" s="1">
-        <v>204</v>
+        <v>452</v>
       </c>
       <c r="I27" s="1">
-        <v>208</v>
+        <v>565</v>
       </c>
       <c r="J27" s="1">
-        <v>-4</v>
+        <v>-113</v>
       </c>
       <c r="K27" s="2">
-        <v>0.47599999999999998</v>
+        <v>0.25900000000000001</v>
       </c>
       <c r="L27" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M27" s="1">
         <v>0</v>
       </c>
       <c r="N27" s="1">
-        <v>4</v>
-      </c>
-      <c r="O27" s="13">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="P27" s="1"/>
-      <c r="Q27" s="4"/>
+        <v>7</v>
+      </c>
+      <c r="O27" s="8">
+        <f t="shared" si="0"/>
+        <v>8.4</v>
+      </c>
+      <c r="P27" s="1">
+        <v>1</v>
+      </c>
+      <c r="Q27" s="6">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
       <c r="R27" s="1"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>26</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="D28" s="1">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="E28" s="1">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F28" s="1">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G28" s="1">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="H28" s="1">
-        <v>333</v>
+        <v>440</v>
       </c>
       <c r="I28" s="1">
-        <v>322</v>
+        <v>464</v>
       </c>
       <c r="J28" s="1">
-        <v>11</v>
+        <v>-24</v>
       </c>
       <c r="K28" s="2">
-        <v>0.51500000000000001</v>
+        <v>0.54500000000000004</v>
       </c>
       <c r="L28" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M28" s="1">
         <v>1</v>
@@ -2768,14 +2788,14 @@
       <c r="N28" s="1">
         <v>2</v>
       </c>
-      <c r="O28" s="13">
-        <f t="shared" si="0"/>
-        <v>10.333333333333334</v>
+      <c r="O28" s="8">
+        <f t="shared" si="0"/>
+        <v>10.25</v>
       </c>
       <c r="P28" s="1">
         <v>0</v>
       </c>
-      <c r="Q28" s="4">
+      <c r="Q28" s="6">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2785,38 +2805,38 @@
       <c r="A29" s="1">
         <v>26</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D29" s="1">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="E29" s="1">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F29" s="1">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G29" s="1">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="H29" s="1">
-        <v>304</v>
+        <v>413</v>
       </c>
       <c r="I29" s="1">
-        <v>322</v>
+        <v>431</v>
       </c>
       <c r="J29" s="1">
         <v>-18</v>
       </c>
       <c r="K29" s="2">
-        <v>0.40600000000000003</v>
+        <v>0.41899999999999998</v>
       </c>
       <c r="L29" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M29" s="1">
         <v>0</v>
@@ -2824,14 +2844,14 @@
       <c r="N29" s="1">
         <v>4</v>
       </c>
-      <c r="O29" s="13">
-        <f t="shared" si="0"/>
-        <v>10.333333333333334</v>
+      <c r="O29" s="8">
+        <f t="shared" si="0"/>
+        <v>10.25</v>
       </c>
       <c r="P29" s="1">
         <v>0</v>
       </c>
-      <c r="Q29" s="4">
+      <c r="Q29" s="6">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -2839,7 +2859,7 @@
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>39</v>
@@ -2848,28 +2868,28 @@
         <v>8</v>
       </c>
       <c r="D30" s="1">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E30" s="1">
         <v>10</v>
       </c>
       <c r="F30" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G30" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H30" s="1">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="I30" s="1">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="J30" s="1">
-        <v>2</v>
+        <v>-4</v>
       </c>
       <c r="K30" s="2">
-        <v>0.45500000000000002</v>
+        <v>0.47599999999999998</v>
       </c>
       <c r="L30" s="1">
         <v>2</v>
@@ -2878,19 +2898,14 @@
         <v>0</v>
       </c>
       <c r="N30" s="1">
-        <v>9</v>
-      </c>
-      <c r="O30" s="13">
-        <f t="shared" si="0"/>
-        <v>15.5</v>
-      </c>
-      <c r="P30" s="1">
-        <v>2</v>
-      </c>
-      <c r="Q30" s="8">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="O30" s="8">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="6"/>
       <c r="R30" s="1"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
@@ -2904,28 +2919,28 @@
         <v>8</v>
       </c>
       <c r="D31" s="1">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E31" s="1">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F31" s="1">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G31" s="1">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H31" s="1">
-        <v>300</v>
+        <v>322</v>
       </c>
       <c r="I31" s="1">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="J31" s="1">
-        <v>-15</v>
+        <v>2</v>
       </c>
       <c r="K31" s="2">
-        <v>0.40600000000000003</v>
+        <v>0.48499999999999999</v>
       </c>
       <c r="L31" s="1">
         <v>3</v>
@@ -2934,70 +2949,70 @@
         <v>0</v>
       </c>
       <c r="N31" s="1">
-        <v>5</v>
-      </c>
-      <c r="O31" s="13">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="P31" s="1">
-        <v>1</v>
-      </c>
-      <c r="Q31" s="4">
-        <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="O31" s="8">
+        <f t="shared" si="0"/>
+        <v>10.333333333333334</v>
+      </c>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="6"/>
       <c r="R31" s="1"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>30</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="5" t="s">
         <v>41</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D32" s="1">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E32" s="1">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F32" s="1">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G32" s="1">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="H32" s="1">
-        <v>224</v>
+        <v>300</v>
       </c>
       <c r="I32" s="1">
-        <v>233</v>
+        <v>315</v>
       </c>
       <c r="J32" s="1">
-        <v>-9</v>
+        <v>-15</v>
       </c>
       <c r="K32" s="2">
-        <v>0.45500000000000002</v>
+        <v>0.40600000000000003</v>
       </c>
       <c r="L32" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M32" s="1">
         <v>0</v>
       </c>
       <c r="N32" s="1">
-        <v>9</v>
-      </c>
-      <c r="O32" s="13">
-        <f t="shared" si="0"/>
-        <v>14.5</v>
-      </c>
-      <c r="P32" s="1"/>
-      <c r="Q32" s="4"/>
+        <v>5</v>
+      </c>
+      <c r="O32" s="8">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="P32" s="1">
+        <v>1</v>
+      </c>
+      <c r="Q32" s="6">
+        <f t="shared" si="1"/>
+        <v>0.33333333333333331</v>
+      </c>
       <c r="R32" s="1"/>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
@@ -3008,47 +3023,47 @@
         <v>42</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="D33" s="1">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E33" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F33" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G33" s="1">
         <v>22</v>
       </c>
       <c r="H33" s="1">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="I33" s="1">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="J33" s="1">
-        <v>-6</v>
+        <v>-9</v>
       </c>
       <c r="K33" s="2">
-        <v>0.40899999999999997</v>
+        <v>0.45500000000000002</v>
       </c>
       <c r="L33" s="1">
         <v>2</v>
       </c>
       <c r="M33" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N33" s="1">
-        <v>3</v>
-      </c>
-      <c r="O33" s="13">
-        <f t="shared" si="0"/>
-        <v>13</v>
+        <v>9</v>
+      </c>
+      <c r="O33" s="8">
+        <f t="shared" si="0"/>
+        <v>14.5</v>
       </c>
       <c r="P33" s="1"/>
-      <c r="Q33" s="4"/>
+      <c r="Q33" s="6"/>
       <c r="R33" s="1"/>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
@@ -3059,108 +3074,108 @@
         <v>43</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="D34" s="1">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="E34" s="1">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F34" s="1">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G34" s="1">
         <v>22</v>
       </c>
       <c r="H34" s="1">
-        <v>235</v>
+        <v>219</v>
       </c>
       <c r="I34" s="1">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="J34" s="1">
-        <v>8</v>
-      </c>
-      <c r="K34" s="3">
-        <v>0.5</v>
+        <v>-6</v>
+      </c>
+      <c r="K34" s="2">
+        <v>0.40899999999999997</v>
       </c>
       <c r="L34" s="1">
         <v>2</v>
       </c>
       <c r="M34" s="1">
+        <v>1</v>
+      </c>
+      <c r="N34" s="1">
+        <v>3</v>
+      </c>
+      <c r="O34" s="8">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="P34" s="1"/>
+      <c r="Q34" s="6"/>
+      <c r="R34" s="1"/>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>33</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" s="1">
+        <v>21</v>
+      </c>
+      <c r="E35" s="1">
+        <v>11</v>
+      </c>
+      <c r="F35" s="1">
+        <v>11</v>
+      </c>
+      <c r="G35" s="1">
+        <v>22</v>
+      </c>
+      <c r="H35" s="1">
+        <v>235</v>
+      </c>
+      <c r="I35" s="1">
+        <v>227</v>
+      </c>
+      <c r="J35" s="1">
+        <v>8</v>
+      </c>
+      <c r="K35" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="L35" s="1">
+        <v>2</v>
+      </c>
+      <c r="M35" s="1">
         <v>0</v>
       </c>
-      <c r="N34" s="1">
+      <c r="N35" s="1">
         <v>6</v>
       </c>
-      <c r="O34" s="13">
+      <c r="O35" s="8">
         <f t="shared" si="0"/>
         <v>10.5</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P35" s="1">
         <v>0</v>
       </c>
-      <c r="Q34" s="4">
+      <c r="Q35" s="6">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="R34" s="1"/>
-    </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
-        <v>32</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D35" s="1">
-        <v>21</v>
-      </c>
-      <c r="E35" s="1">
-        <v>11</v>
-      </c>
-      <c r="F35" s="1">
-        <v>11</v>
-      </c>
-      <c r="G35" s="1">
-        <v>22</v>
-      </c>
-      <c r="H35" s="1">
-        <v>215</v>
-      </c>
-      <c r="I35" s="1">
-        <v>212</v>
-      </c>
-      <c r="J35" s="1">
-        <v>3</v>
-      </c>
-      <c r="K35" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="L35" s="1">
-        <v>2</v>
-      </c>
-      <c r="M35" s="1">
-        <v>0</v>
-      </c>
-      <c r="N35" s="1">
-        <v>4</v>
-      </c>
-      <c r="O35" s="13">
-        <f t="shared" si="0"/>
-        <v>10.5</v>
-      </c>
-      <c r="P35" s="1"/>
-      <c r="Q35" s="4"/>
       <c r="R35" s="1"/>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>45</v>
@@ -3201,23 +3216,23 @@
       <c r="N36" s="1">
         <v>2</v>
       </c>
-      <c r="O36" s="13">
+      <c r="O36" s="8">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="P36" s="1"/>
-      <c r="Q36" s="4"/>
+      <c r="Q36" s="6"/>
       <c r="R36" s="1"/>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D37" s="1">
         <v>21</v>
@@ -3252,12 +3267,12 @@
       <c r="N37" s="1">
         <v>2</v>
       </c>
-      <c r="O37" s="13">
+      <c r="O37" s="8">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="P37" s="1"/>
-      <c r="Q37" s="4"/>
+      <c r="Q37" s="6"/>
       <c r="R37" s="1"/>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
@@ -3303,12 +3318,12 @@
       <c r="N38" s="1">
         <v>3</v>
       </c>
-      <c r="O38" s="13">
+      <c r="O38" s="8">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="P38" s="1"/>
-      <c r="Q38" s="4"/>
+      <c r="Q38" s="6"/>
       <c r="R38" s="1"/>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
@@ -3325,25 +3340,25 @@
         <v>17</v>
       </c>
       <c r="E39" s="1">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F39" s="1">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G39" s="1">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H39" s="1">
-        <v>209</v>
+        <v>180</v>
       </c>
       <c r="I39" s="1">
-        <v>232</v>
+        <v>194</v>
       </c>
       <c r="J39" s="1">
-        <v>-23</v>
+        <v>-14</v>
       </c>
       <c r="K39" s="2">
-        <v>0.27300000000000002</v>
+        <v>0.47399999999999998</v>
       </c>
       <c r="L39" s="1">
         <v>2</v>
@@ -3352,14 +3367,14 @@
         <v>0</v>
       </c>
       <c r="N39" s="1">
-        <v>9</v>
-      </c>
-      <c r="O39" s="13">
+        <v>7</v>
+      </c>
+      <c r="O39" s="8">
         <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
       <c r="P39" s="1"/>
-      <c r="Q39" s="4"/>
+      <c r="Q39" s="6"/>
       <c r="R39" s="1"/>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
@@ -3379,73 +3394,73 @@
         <v>6</v>
       </c>
       <c r="F40" s="1">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="G40" s="1">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="H40" s="1">
-        <v>110</v>
+        <v>209</v>
       </c>
       <c r="I40" s="1">
-        <v>82</v>
+        <v>232</v>
       </c>
       <c r="J40" s="1">
-        <v>28</v>
+        <v>-23</v>
       </c>
       <c r="K40" s="2">
-        <v>0.54500000000000004</v>
+        <v>0.27300000000000002</v>
       </c>
       <c r="L40" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M40" s="1">
         <v>0</v>
       </c>
       <c r="N40" s="1">
-        <v>6</v>
-      </c>
-      <c r="O40" s="13">
-        <f t="shared" si="0"/>
-        <v>17</v>
+        <v>9</v>
+      </c>
+      <c r="O40" s="8">
+        <f t="shared" si="0"/>
+        <v>8.5</v>
       </c>
       <c r="P40" s="1"/>
-      <c r="Q40" s="4"/>
+      <c r="Q40" s="6"/>
       <c r="R40" s="1"/>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="D41" s="1">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E41" s="1">
+        <v>6</v>
+      </c>
+      <c r="F41" s="1">
         <v>5</v>
-      </c>
-      <c r="F41" s="1">
-        <v>6</v>
       </c>
       <c r="G41" s="1">
         <v>11</v>
       </c>
       <c r="H41" s="1">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I41" s="1">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="J41" s="1">
-        <v>-1</v>
+        <v>28</v>
       </c>
       <c r="K41" s="2">
-        <v>0.45500000000000002</v>
+        <v>0.54500000000000004</v>
       </c>
       <c r="L41" s="1">
         <v>1</v>
@@ -3454,49 +3469,49 @@
         <v>0</v>
       </c>
       <c r="N41" s="1">
-        <v>8</v>
-      </c>
-      <c r="O41" s="13">
-        <f t="shared" si="0"/>
-        <v>16</v>
+        <v>6</v>
+      </c>
+      <c r="O41" s="8">
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
       <c r="P41" s="1"/>
-      <c r="Q41" s="4"/>
+      <c r="Q41" s="6"/>
       <c r="R41" s="1"/>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>51</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="D42" s="1">
         <v>16</v>
       </c>
       <c r="E42" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F42" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G42" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H42" s="1">
-        <v>93</v>
+        <v>113</v>
       </c>
       <c r="I42" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="J42" s="1">
-        <v>-11</v>
-      </c>
-      <c r="K42" s="3">
-        <v>0.3</v>
+        <v>-1</v>
+      </c>
+      <c r="K42" s="2">
+        <v>0.45500000000000002</v>
       </c>
       <c r="L42" s="1">
         <v>1</v>
@@ -3505,65 +3520,65 @@
         <v>0</v>
       </c>
       <c r="N42" s="1">
-        <v>9</v>
-      </c>
-      <c r="O42" s="13">
+        <v>8</v>
+      </c>
+      <c r="O42" s="8">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="P42" s="1"/>
-      <c r="Q42" s="4"/>
+      <c r="Q42" s="6"/>
       <c r="R42" s="1"/>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>52</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="D43" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E43" s="1">
+        <v>3</v>
+      </c>
+      <c r="F43" s="1">
+        <v>7</v>
+      </c>
+      <c r="G43" s="1">
+        <v>10</v>
+      </c>
+      <c r="H43" s="1">
+        <v>93</v>
+      </c>
+      <c r="I43" s="1">
+        <v>104</v>
+      </c>
+      <c r="J43" s="1">
+        <v>-11</v>
+      </c>
+      <c r="K43" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="L43" s="1">
+        <v>1</v>
+      </c>
+      <c r="M43" s="1">
+        <v>0</v>
+      </c>
+      <c r="N43" s="1">
         <v>9</v>
       </c>
-      <c r="F43" s="1">
-        <v>2</v>
-      </c>
-      <c r="G43" s="1">
-        <v>11</v>
-      </c>
-      <c r="H43" s="1">
-        <v>118</v>
-      </c>
-      <c r="I43" s="1">
-        <v>87</v>
-      </c>
-      <c r="J43" s="1">
-        <v>31</v>
-      </c>
-      <c r="K43" s="2">
-        <v>0.81799999999999995</v>
-      </c>
-      <c r="L43" s="1">
-        <v>1</v>
-      </c>
-      <c r="M43" s="1">
-        <v>1</v>
-      </c>
-      <c r="N43" s="1">
-        <v>1</v>
-      </c>
-      <c r="O43" s="13">
-        <f t="shared" si="0"/>
-        <v>14</v>
+      <c r="O43" s="8">
+        <f t="shared" si="0"/>
+        <v>16</v>
       </c>
       <c r="P43" s="1"/>
-      <c r="Q43" s="4"/>
+      <c r="Q43" s="6"/>
       <c r="R43" s="1"/>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
@@ -3577,28 +3592,28 @@
         <v>8</v>
       </c>
       <c r="D44" s="1">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E44" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F44" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G44" s="1">
         <v>11</v>
       </c>
       <c r="H44" s="1">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="I44" s="1">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="J44" s="1">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="K44" s="2">
-        <v>0.63600000000000001</v>
+        <v>0.81799999999999995</v>
       </c>
       <c r="L44" s="1">
         <v>1</v>
@@ -3607,15 +3622,17 @@
         <v>1</v>
       </c>
       <c r="N44" s="1">
-        <v>2</v>
-      </c>
-      <c r="O44" s="13">
-        <f t="shared" si="0"/>
-        <v>13</v>
+        <v>1</v>
+      </c>
+      <c r="O44" s="8">
+        <f t="shared" si="0"/>
+        <v>14</v>
       </c>
       <c r="P44" s="1"/>
-      <c r="Q44" s="4"/>
-      <c r="R44" s="1"/>
+      <c r="Q44" s="6"/>
+      <c r="R44" s="1">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
@@ -3628,7 +3645,7 @@
         <v>8</v>
       </c>
       <c r="D45" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E45" s="1">
         <v>7</v>
@@ -3640,13 +3657,13 @@
         <v>11</v>
       </c>
       <c r="H45" s="1">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="I45" s="1">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J45" s="1">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K45" s="2">
         <v>0.63600000000000001</v>
@@ -3658,19 +3675,19 @@
         <v>1</v>
       </c>
       <c r="N45" s="1">
-        <v>3</v>
-      </c>
-      <c r="O45" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
+        <v>2</v>
+      </c>
+      <c r="O45" s="8">
+        <f t="shared" si="0"/>
+        <v>13</v>
       </c>
       <c r="P45" s="1"/>
-      <c r="Q45" s="4"/>
+      <c r="Q45" s="6"/>
       <c r="R45" s="1"/>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>55</v>
@@ -3682,52 +3699,52 @@
         <v>12</v>
       </c>
       <c r="E46" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F46" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G46" s="1">
         <v>11</v>
       </c>
       <c r="H46" s="1">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="I46" s="1">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J46" s="1">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="K46" s="2">
-        <v>0.54500000000000004</v>
+        <v>0.63600000000000001</v>
       </c>
       <c r="L46" s="1">
         <v>1</v>
       </c>
       <c r="M46" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N46" s="1">
-        <v>4</v>
-      </c>
-      <c r="O46" s="13">
+        <v>3</v>
+      </c>
+      <c r="O46" s="8">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="P46" s="1"/>
-      <c r="Q46" s="4"/>
+      <c r="Q46" s="6"/>
       <c r="R46" s="1"/>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="D47" s="1">
         <v>12</v>
@@ -3762,26 +3779,26 @@
       <c r="N47" s="1">
         <v>4</v>
       </c>
-      <c r="O47" s="13">
+      <c r="O47" s="8">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="P47" s="1"/>
-      <c r="Q47" s="4"/>
+      <c r="Q47" s="6"/>
       <c r="R47" s="1"/>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="D48" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E48" s="1">
         <v>6</v>
@@ -3793,13 +3810,13 @@
         <v>11</v>
       </c>
       <c r="H48" s="1">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="I48" s="1">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="J48" s="1">
-        <v>-6</v>
+        <v>9</v>
       </c>
       <c r="K48" s="2">
         <v>0.54500000000000004</v>
@@ -3811,14 +3828,14 @@
         <v>0</v>
       </c>
       <c r="N48" s="1">
-        <v>5</v>
-      </c>
-      <c r="O48" s="13">
-        <f t="shared" si="0"/>
-        <v>11</v>
+        <v>4</v>
+      </c>
+      <c r="O48" s="8">
+        <f t="shared" si="0"/>
+        <v>12</v>
       </c>
       <c r="P48" s="1"/>
-      <c r="Q48" s="4"/>
+      <c r="Q48" s="6"/>
       <c r="R48" s="1"/>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.25">
@@ -3826,34 +3843,34 @@
         <v>47</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="D49" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E49" s="1">
+        <v>6</v>
+      </c>
+      <c r="F49" s="1">
         <v>5</v>
-      </c>
-      <c r="F49" s="1">
-        <v>6</v>
       </c>
       <c r="G49" s="1">
         <v>11</v>
       </c>
       <c r="H49" s="1">
+        <v>104</v>
+      </c>
+      <c r="I49" s="1">
         <v>110</v>
       </c>
-      <c r="I49" s="1">
-        <v>115</v>
-      </c>
       <c r="J49" s="1">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="K49" s="2">
-        <v>0.45500000000000002</v>
+        <v>0.54500000000000004</v>
       </c>
       <c r="L49" s="1">
         <v>1</v>
@@ -3862,49 +3879,49 @@
         <v>0</v>
       </c>
       <c r="N49" s="1">
-        <v>7</v>
-      </c>
-      <c r="O49" s="13">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <v>5</v>
+      </c>
+      <c r="O49" s="8">
+        <f t="shared" si="0"/>
+        <v>11</v>
       </c>
       <c r="P49" s="1"/>
-      <c r="Q49" s="4"/>
+      <c r="Q49" s="6"/>
       <c r="R49" s="1"/>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>58</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="D50" s="1">
         <v>10</v>
       </c>
       <c r="E50" s="1">
+        <v>5</v>
+      </c>
+      <c r="F50" s="1">
         <v>6</v>
-      </c>
-      <c r="F50" s="1">
-        <v>5</v>
       </c>
       <c r="G50" s="1">
         <v>11</v>
       </c>
       <c r="H50" s="1">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="I50" s="1">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="J50" s="1">
-        <v>2</v>
+        <v>-5</v>
       </c>
       <c r="K50" s="2">
-        <v>0.54500000000000004</v>
+        <v>0.45500000000000002</v>
       </c>
       <c r="L50" s="1">
         <v>1</v>
@@ -3915,23 +3932,23 @@
       <c r="N50" s="1">
         <v>7</v>
       </c>
-      <c r="O50" s="13">
+      <c r="O50" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="P50" s="1"/>
-      <c r="Q50" s="4"/>
+      <c r="Q50" s="6"/>
       <c r="R50" s="1"/>
     </row>
     <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>59</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D51" s="1">
         <v>10</v>
@@ -3966,23 +3983,23 @@
       <c r="N51" s="1">
         <v>8</v>
       </c>
-      <c r="O51" s="13">
+      <c r="O51" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="P51" s="1"/>
-      <c r="Q51" s="4"/>
+      <c r="Q51" s="6"/>
       <c r="R51" s="1"/>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>60</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D52" s="1">
         <v>10</v>
@@ -4017,17 +4034,17 @@
       <c r="N52" s="1">
         <v>8</v>
       </c>
-      <c r="O52" s="13">
+      <c r="O52" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="P52" s="1"/>
-      <c r="Q52" s="4"/>
+      <c r="Q52" s="6"/>
       <c r="R52" s="1"/>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>61</v>
@@ -4068,12 +4085,12 @@
       <c r="N53" s="1">
         <v>7</v>
       </c>
-      <c r="O53" s="13">
+      <c r="O53" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="P53" s="1"/>
-      <c r="Q53" s="4"/>
+      <c r="Q53" s="6"/>
       <c r="R53" s="1"/>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.25">
@@ -4084,7 +4101,7 @@
         <v>62</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D54" s="1">
         <v>9</v>
@@ -4119,47 +4136,47 @@
       <c r="N54" s="1">
         <v>10</v>
       </c>
-      <c r="O54" s="13">
+      <c r="O54" s="8">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="P54" s="1"/>
-      <c r="Q54" s="4"/>
+      <c r="Q54" s="6"/>
       <c r="R54" s="1"/>
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>63</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="D55" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E55" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F55" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G55" s="1">
         <v>11</v>
       </c>
       <c r="H55" s="1">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="I55" s="1">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="J55" s="1">
-        <v>-11</v>
+        <v>-3</v>
       </c>
       <c r="K55" s="2">
-        <v>0.27300000000000002</v>
+        <v>0.36399999999999999</v>
       </c>
       <c r="L55" s="1">
         <v>1</v>
@@ -4168,22 +4185,22 @@
         <v>0</v>
       </c>
       <c r="N55" s="1">
-        <v>12</v>
-      </c>
-      <c r="O55" s="13">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="O55" s="8">
+        <f t="shared" si="0"/>
+        <v>9</v>
       </c>
       <c r="P55" s="1"/>
-      <c r="Q55" s="4"/>
+      <c r="Q55" s="6"/>
       <c r="R55" s="1"/>
     </row>
     <row r="56" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>8</v>
@@ -4192,25 +4209,25 @@
         <v>8</v>
       </c>
       <c r="E56" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F56" s="1">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G56" s="1">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H56" s="1">
-        <v>23</v>
+        <v>107</v>
       </c>
       <c r="I56" s="1">
-        <v>22</v>
+        <v>118</v>
       </c>
       <c r="J56" s="1">
-        <v>1</v>
-      </c>
-      <c r="K56" s="3">
-        <v>0.5</v>
+        <v>-11</v>
+      </c>
+      <c r="K56" s="2">
+        <v>0.27300000000000002</v>
       </c>
       <c r="L56" s="1">
         <v>1</v>
@@ -4221,13 +4238,64 @@
       <c r="N56" s="1">
         <v>12</v>
       </c>
-      <c r="O56" s="13">
+      <c r="O56" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="P56" s="1"/>
-      <c r="Q56" s="4"/>
+      <c r="Q56" s="6"/>
       <c r="R56" s="1"/>
+    </row>
+    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>54</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" s="1">
+        <v>8</v>
+      </c>
+      <c r="E57" s="1">
+        <v>1</v>
+      </c>
+      <c r="F57" s="1">
+        <v>1</v>
+      </c>
+      <c r="G57" s="1">
+        <v>2</v>
+      </c>
+      <c r="H57" s="1">
+        <v>23</v>
+      </c>
+      <c r="I57" s="1">
+        <v>22</v>
+      </c>
+      <c r="J57" s="1">
+        <v>1</v>
+      </c>
+      <c r="K57" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="L57" s="1">
+        <v>1</v>
+      </c>
+      <c r="M57" s="1">
+        <v>0</v>
+      </c>
+      <c r="N57" s="1">
+        <v>12</v>
+      </c>
+      <c r="O57" s="8">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="P57" s="1"/>
+      <c r="Q57" s="6"/>
+      <c r="R57" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>